<commit_message>
Evidencia del 28 de septiembre
</commit_message>
<xml_diff>
--- a/Cronograma/Itinerario-Ayo_Alisson V3.xlsx
+++ b/Cronograma/Itinerario-Ayo_Alisson V3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Desktop\Prácticas\37009_PPP\Cronograma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BE9CAC7-DEB0-49ED-A5D7-0AC70E096BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9869C85-39E0-46EC-9244-8F4D8963318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -884,68 +884,68 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1240,15 +1240,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.7">
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
@@ -1316,10 +1316,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="26">
+      <c r="A9" s="33">
         <v>46279</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="33" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="14" t="s">
@@ -1329,17 +1329,17 @@
         <v>2</v>
       </c>
       <c r="E9" s="14"/>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="28">
-        <v>6</v>
-      </c>
-      <c r="H9" s="24"/>
+      <c r="G9" s="35">
+        <v>6</v>
+      </c>
+      <c r="H9" s="43"/>
     </row>
     <row r="10" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
+      <c r="A10" s="33"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="14" t="s">
         <v>19</v>
       </c>
@@ -1347,13 +1347,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="14"/>
-      <c r="F10" s="27"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="24"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="43"/>
     </row>
     <row r="11" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A11" s="26"/>
-      <c r="B11" s="26"/>
+      <c r="A11" s="33"/>
+      <c r="B11" s="33"/>
       <c r="C11" s="14" t="s">
         <v>20</v>
       </c>
@@ -1364,15 +1364,15 @@
         <f>SUM(D9:D11)</f>
         <v>6</v>
       </c>
-      <c r="F11" s="27"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="24"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="43"/>
     </row>
     <row r="12" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A12" s="26">
+      <c r="A12" s="33">
         <v>46280</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="33" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1382,17 +1382,17 @@
         <v>2</v>
       </c>
       <c r="E12" s="14"/>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="34" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="28">
-        <v>6</v>
-      </c>
-      <c r="H12" s="24"/>
+      <c r="G12" s="35">
+        <v>6</v>
+      </c>
+      <c r="H12" s="43"/>
     </row>
     <row r="13" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A13" s="26"/>
-      <c r="B13" s="26"/>
+      <c r="A13" s="33"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="14" t="s">
         <v>24</v>
       </c>
@@ -1400,13 +1400,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="13"/>
-      <c r="F13" s="27"/>
-      <c r="G13" s="28"/>
-      <c r="H13" s="24"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="35"/>
+      <c r="H13" s="43"/>
     </row>
     <row r="14" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A14" s="26"/>
-      <c r="B14" s="26"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="33"/>
       <c r="C14" s="14" t="s">
         <v>21</v>
       </c>
@@ -1416,15 +1416,15 @@
       <c r="E14" s="14">
         <v>6</v>
       </c>
-      <c r="F14" s="27"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="24"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="43"/>
     </row>
     <row r="15" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A15" s="26">
+      <c r="A15" s="33">
         <v>46281</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="33" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -1434,17 +1434,17 @@
         <v>2</v>
       </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="27" t="s">
+      <c r="F15" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="28">
-        <v>6</v>
-      </c>
-      <c r="H15" s="24"/>
+      <c r="G15" s="35">
+        <v>6</v>
+      </c>
+      <c r="H15" s="43"/>
     </row>
     <row r="16" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A16" s="26"/>
-      <c r="B16" s="26"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="33"/>
       <c r="C16" s="20" t="s">
         <v>27</v>
       </c>
@@ -1452,13 +1452,13 @@
         <v>2</v>
       </c>
       <c r="E16" s="13"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="28"/>
-      <c r="H16" s="24"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="43"/>
     </row>
     <row r="17" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A17" s="26"/>
-      <c r="B17" s="26"/>
+      <c r="A17" s="33"/>
+      <c r="B17" s="33"/>
       <c r="C17" s="20" t="s">
         <v>28</v>
       </c>
@@ -1468,15 +1468,15 @@
       <c r="E17" s="14">
         <v>6</v>
       </c>
-      <c r="F17" s="27"/>
-      <c r="G17" s="28"/>
-      <c r="H17" s="24"/>
+      <c r="F17" s="34"/>
+      <c r="G17" s="35"/>
+      <c r="H17" s="43"/>
     </row>
     <row r="18" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A18" s="26">
+      <c r="A18" s="33">
         <v>46282</v>
       </c>
-      <c r="B18" s="26" t="s">
+      <c r="B18" s="33" t="s">
         <v>29</v>
       </c>
       <c r="C18" s="14" t="s">
@@ -1486,17 +1486,17 @@
         <v>2</v>
       </c>
       <c r="E18" s="13"/>
-      <c r="F18" s="27" t="s">
+      <c r="F18" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="28">
-        <v>6</v>
-      </c>
-      <c r="H18" s="24"/>
+      <c r="G18" s="35">
+        <v>6</v>
+      </c>
+      <c r="H18" s="43"/>
     </row>
     <row r="19" spans="1:8" ht="38.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="26"/>
-      <c r="B19" s="26"/>
+      <c r="A19" s="33"/>
+      <c r="B19" s="33"/>
       <c r="C19" s="14" t="s">
         <v>31</v>
       </c>
@@ -1504,13 +1504,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="13"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="28"/>
-      <c r="H19" s="24"/>
+      <c r="F19" s="34"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="43"/>
     </row>
     <row r="20" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A20" s="26"/>
-      <c r="B20" s="26"/>
+      <c r="A20" s="33"/>
+      <c r="B20" s="33"/>
       <c r="C20" s="14" t="s">
         <v>32</v>
       </c>
@@ -1520,15 +1520,15 @@
       <c r="E20" s="14">
         <v>6</v>
       </c>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="24"/>
+      <c r="F20" s="34"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="43"/>
     </row>
     <row r="21" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A21" s="26">
+      <c r="A21" s="33">
         <v>46283</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="B21" s="33" t="s">
         <v>33</v>
       </c>
       <c r="C21" s="14" t="s">
@@ -1538,17 +1538,17 @@
         <v>2</v>
       </c>
       <c r="E21" s="13"/>
-      <c r="F21" s="27" t="s">
+      <c r="F21" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="28">
-        <v>6</v>
-      </c>
-      <c r="H21" s="24"/>
+      <c r="G21" s="35">
+        <v>6</v>
+      </c>
+      <c r="H21" s="43"/>
     </row>
     <row r="22" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A22" s="26"/>
-      <c r="B22" s="26"/>
+      <c r="A22" s="33"/>
+      <c r="B22" s="33"/>
       <c r="C22" s="14" t="s">
         <v>35</v>
       </c>
@@ -1556,13 +1556,13 @@
         <v>2</v>
       </c>
       <c r="E22" s="13"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28"/>
-      <c r="H22" s="24"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="35"/>
+      <c r="H22" s="43"/>
     </row>
     <row r="23" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A23" s="26"/>
-      <c r="B23" s="26"/>
+      <c r="A23" s="33"/>
+      <c r="B23" s="33"/>
       <c r="C23" s="14" t="s">
         <v>36</v>
       </c>
@@ -1572,15 +1572,15 @@
       <c r="E23" s="14">
         <v>6</v>
       </c>
-      <c r="F23" s="27"/>
-      <c r="G23" s="28"/>
-      <c r="H23" s="24"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="43"/>
     </row>
     <row r="24" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A24" s="26">
+      <c r="A24" s="33">
         <v>46286</v>
       </c>
-      <c r="B24" s="26" t="s">
+      <c r="B24" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="14" t="s">
@@ -1590,17 +1590,17 @@
         <v>2</v>
       </c>
       <c r="E24" s="14"/>
-      <c r="F24" s="27" t="s">
+      <c r="F24" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="G24" s="28">
-        <v>6</v>
-      </c>
-      <c r="H24" s="24"/>
+      <c r="G24" s="35">
+        <v>6</v>
+      </c>
+      <c r="H24" s="43"/>
     </row>
     <row r="25" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A25" s="26"/>
-      <c r="B25" s="26"/>
+      <c r="A25" s="33"/>
+      <c r="B25" s="33"/>
       <c r="C25" s="14" t="s">
         <v>39</v>
       </c>
@@ -1608,13 +1608,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="13"/>
-      <c r="F25" s="27"/>
-      <c r="G25" s="28"/>
-      <c r="H25" s="24"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="43"/>
     </row>
     <row r="26" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A26" s="26"/>
-      <c r="B26" s="26"/>
+      <c r="A26" s="33"/>
+      <c r="B26" s="33"/>
       <c r="C26" s="14" t="s">
         <v>40</v>
       </c>
@@ -1624,15 +1624,15 @@
       <c r="E26" s="14">
         <v>6</v>
       </c>
-      <c r="F26" s="27"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="24"/>
+      <c r="F26" s="34"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="43"/>
     </row>
     <row r="27" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A27" s="26">
+      <c r="A27" s="33">
         <v>46287</v>
       </c>
-      <c r="B27" s="26" t="s">
+      <c r="B27" s="33" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -1642,17 +1642,17 @@
         <v>2</v>
       </c>
       <c r="E27" s="13"/>
-      <c r="F27" s="27" t="s">
+      <c r="F27" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="28">
-        <v>6</v>
-      </c>
-      <c r="H27" s="24"/>
+      <c r="G27" s="35">
+        <v>6</v>
+      </c>
+      <c r="H27" s="43"/>
     </row>
     <row r="28" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A28" s="26"/>
-      <c r="B28" s="26"/>
+      <c r="A28" s="33"/>
+      <c r="B28" s="33"/>
       <c r="C28" s="14" t="s">
         <v>43</v>
       </c>
@@ -1660,13 +1660,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="13"/>
-      <c r="F28" s="27"/>
-      <c r="G28" s="28"/>
-      <c r="H28" s="24"/>
+      <c r="F28" s="34"/>
+      <c r="G28" s="35"/>
+      <c r="H28" s="43"/>
     </row>
     <row r="29" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A29" s="26"/>
-      <c r="B29" s="26"/>
+      <c r="A29" s="33"/>
+      <c r="B29" s="33"/>
       <c r="C29" s="14" t="s">
         <v>44</v>
       </c>
@@ -1676,15 +1676,15 @@
       <c r="E29" s="14">
         <v>6</v>
       </c>
-      <c r="F29" s="27"/>
-      <c r="G29" s="28"/>
-      <c r="H29" s="24"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="35"/>
+      <c r="H29" s="43"/>
     </row>
     <row r="30" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A30" s="26">
+      <c r="A30" s="33">
         <v>46288</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="33" t="s">
         <v>45</v>
       </c>
       <c r="C30" s="14" t="s">
@@ -1694,17 +1694,17 @@
         <v>2</v>
       </c>
       <c r="E30" s="13"/>
-      <c r="F30" s="27" t="s">
+      <c r="F30" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="G30" s="28">
-        <v>6</v>
-      </c>
-      <c r="H30" s="24"/>
+      <c r="G30" s="35">
+        <v>6</v>
+      </c>
+      <c r="H30" s="43"/>
     </row>
     <row r="31" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A31" s="26"/>
-      <c r="B31" s="26"/>
+      <c r="A31" s="33"/>
+      <c r="B31" s="33"/>
       <c r="C31" s="14" t="s">
         <v>47</v>
       </c>
@@ -1712,13 +1712,13 @@
         <v>2</v>
       </c>
       <c r="E31" s="13"/>
-      <c r="F31" s="27"/>
-      <c r="G31" s="28"/>
-      <c r="H31" s="24"/>
+      <c r="F31" s="34"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="43"/>
     </row>
     <row r="32" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A32" s="26"/>
-      <c r="B32" s="26"/>
+      <c r="A32" s="33"/>
+      <c r="B32" s="33"/>
       <c r="C32" s="14" t="s">
         <v>48</v>
       </c>
@@ -1728,15 +1728,15 @@
       <c r="E32" s="14">
         <v>6</v>
       </c>
-      <c r="F32" s="27"/>
-      <c r="G32" s="28"/>
-      <c r="H32" s="24"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="35"/>
+      <c r="H32" s="43"/>
     </row>
     <row r="33" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A33" s="26">
+      <c r="A33" s="33">
         <v>46289</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="B33" s="33" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="14" t="s">
@@ -1746,17 +1746,17 @@
         <v>2</v>
       </c>
       <c r="E33" s="13"/>
-      <c r="F33" s="27" t="s">
+      <c r="F33" s="34" t="s">
         <v>178</v>
       </c>
-      <c r="G33" s="28">
-        <v>6</v>
-      </c>
-      <c r="H33" s="24"/>
+      <c r="G33" s="35">
+        <v>6</v>
+      </c>
+      <c r="H33" s="43"/>
     </row>
     <row r="34" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A34" s="26"/>
-      <c r="B34" s="26"/>
+      <c r="A34" s="33"/>
+      <c r="B34" s="33"/>
       <c r="C34" s="14" t="s">
         <v>62</v>
       </c>
@@ -1764,13 +1764,13 @@
         <v>2</v>
       </c>
       <c r="E34" s="13"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="28"/>
-      <c r="H34" s="24"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="35"/>
+      <c r="H34" s="43"/>
     </row>
     <row r="35" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="26"/>
-      <c r="B35" s="26"/>
+      <c r="A35" s="33"/>
+      <c r="B35" s="33"/>
       <c r="C35" s="14" t="s">
         <v>63</v>
       </c>
@@ -1780,15 +1780,15 @@
       <c r="E35" s="14">
         <v>6</v>
       </c>
-      <c r="F35" s="27"/>
-      <c r="G35" s="28"/>
-      <c r="H35" s="24"/>
+      <c r="F35" s="34"/>
+      <c r="G35" s="35"/>
+      <c r="H35" s="43"/>
     </row>
     <row r="36" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A36" s="26">
+      <c r="A36" s="33">
         <v>46290</v>
       </c>
-      <c r="B36" s="26" t="s">
+      <c r="B36" s="33" t="s">
         <v>64</v>
       </c>
       <c r="C36" s="14" t="s">
@@ -1798,17 +1798,17 @@
         <v>2</v>
       </c>
       <c r="E36" s="14"/>
-      <c r="F36" s="27" t="s">
+      <c r="F36" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G36" s="28">
-        <v>6</v>
-      </c>
-      <c r="H36" s="24"/>
+      <c r="G36" s="35">
+        <v>6</v>
+      </c>
+      <c r="H36" s="43"/>
     </row>
     <row r="37" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A37" s="26"/>
-      <c r="B37" s="26"/>
+      <c r="A37" s="33"/>
+      <c r="B37" s="33"/>
       <c r="C37" s="14" t="s">
         <v>70</v>
       </c>
@@ -1816,13 +1816,13 @@
         <v>2</v>
       </c>
       <c r="E37" s="13"/>
-      <c r="F37" s="27"/>
-      <c r="G37" s="28"/>
-      <c r="H37" s="24"/>
+      <c r="F37" s="34"/>
+      <c r="G37" s="35"/>
+      <c r="H37" s="43"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A38" s="26"/>
-      <c r="B38" s="26"/>
+      <c r="A38" s="33"/>
+      <c r="B38" s="33"/>
       <c r="C38" s="14" t="s">
         <v>71</v>
       </c>
@@ -1832,15 +1832,15 @@
       <c r="E38" s="14">
         <v>6</v>
       </c>
-      <c r="F38" s="27"/>
-      <c r="G38" s="28"/>
-      <c r="H38" s="24"/>
+      <c r="F38" s="34"/>
+      <c r="G38" s="35"/>
+      <c r="H38" s="43"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A39" s="26">
+      <c r="A39" s="33">
         <v>46293</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="B39" s="33" t="s">
         <v>65</v>
       </c>
       <c r="C39" s="14" t="s">
@@ -1850,17 +1850,17 @@
         <v>2</v>
       </c>
       <c r="E39" s="13"/>
-      <c r="F39" s="27" t="s">
+      <c r="F39" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G39" s="28">
-        <v>6</v>
-      </c>
-      <c r="H39" s="24"/>
+      <c r="G39" s="35">
+        <v>6</v>
+      </c>
+      <c r="H39" s="43"/>
     </row>
     <row r="40" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A40" s="26"/>
-      <c r="B40" s="26"/>
+      <c r="A40" s="33"/>
+      <c r="B40" s="33"/>
       <c r="C40" s="14" t="s">
         <v>73</v>
       </c>
@@ -1868,13 +1868,13 @@
         <v>2</v>
       </c>
       <c r="E40" s="13"/>
-      <c r="F40" s="27"/>
-      <c r="G40" s="28"/>
-      <c r="H40" s="24"/>
+      <c r="F40" s="34"/>
+      <c r="G40" s="35"/>
+      <c r="H40" s="43"/>
     </row>
     <row r="41" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A41" s="26"/>
-      <c r="B41" s="26"/>
+      <c r="A41" s="33"/>
+      <c r="B41" s="33"/>
       <c r="C41" s="14" t="s">
         <v>74</v>
       </c>
@@ -1884,15 +1884,15 @@
       <c r="E41" s="14">
         <v>6</v>
       </c>
-      <c r="F41" s="27"/>
-      <c r="G41" s="28"/>
-      <c r="H41" s="24"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="43"/>
     </row>
     <row r="42" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A42" s="26">
+      <c r="A42" s="33">
         <v>46294</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="B42" s="33" t="s">
         <v>66</v>
       </c>
       <c r="C42" s="14" t="s">
@@ -1902,17 +1902,17 @@
         <v>2</v>
       </c>
       <c r="E42" s="13"/>
-      <c r="F42" s="27" t="s">
+      <c r="F42" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G42" s="28">
-        <v>6</v>
-      </c>
-      <c r="H42" s="24"/>
+      <c r="G42" s="35">
+        <v>6</v>
+      </c>
+      <c r="H42" s="43"/>
     </row>
     <row r="43" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A43" s="26"/>
-      <c r="B43" s="26"/>
+      <c r="A43" s="33"/>
+      <c r="B43" s="33"/>
       <c r="C43" s="14" t="s">
         <v>68</v>
       </c>
@@ -1920,13 +1920,13 @@
         <v>2</v>
       </c>
       <c r="E43" s="13"/>
-      <c r="F43" s="27"/>
-      <c r="G43" s="28"/>
-      <c r="H43" s="24"/>
+      <c r="F43" s="34"/>
+      <c r="G43" s="35"/>
+      <c r="H43" s="43"/>
     </row>
     <row r="44" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A44" s="26"/>
-      <c r="B44" s="26"/>
+      <c r="A44" s="33"/>
+      <c r="B44" s="33"/>
       <c r="C44" s="14" t="s">
         <v>76</v>
       </c>
@@ -1936,15 +1936,15 @@
       <c r="E44" s="14">
         <v>6</v>
       </c>
-      <c r="F44" s="27"/>
-      <c r="G44" s="28"/>
-      <c r="H44" s="24"/>
+      <c r="F44" s="34"/>
+      <c r="G44" s="35"/>
+      <c r="H44" s="43"/>
     </row>
     <row r="45" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A45" s="26">
+      <c r="A45" s="33">
         <v>46295</v>
       </c>
-      <c r="B45" s="26" t="s">
+      <c r="B45" s="33" t="s">
         <v>67</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -1954,17 +1954,17 @@
         <v>2</v>
       </c>
       <c r="E45" s="13"/>
-      <c r="F45" s="27" t="s">
+      <c r="F45" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G45" s="28">
-        <v>6</v>
-      </c>
-      <c r="H45" s="24"/>
+      <c r="G45" s="35">
+        <v>6</v>
+      </c>
+      <c r="H45" s="43"/>
     </row>
     <row r="46" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A46" s="26"/>
-      <c r="B46" s="26"/>
+      <c r="A46" s="33"/>
+      <c r="B46" s="33"/>
       <c r="C46" s="14" t="s">
         <v>78</v>
       </c>
@@ -1972,13 +1972,13 @@
         <v>2</v>
       </c>
       <c r="E46" s="13"/>
-      <c r="F46" s="27"/>
-      <c r="G46" s="28"/>
-      <c r="H46" s="24"/>
+      <c r="F46" s="34"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="43"/>
     </row>
     <row r="47" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A47" s="26"/>
-      <c r="B47" s="26"/>
+      <c r="A47" s="33"/>
+      <c r="B47" s="33"/>
       <c r="C47" s="14" t="s">
         <v>79</v>
       </c>
@@ -1988,15 +1988,15 @@
       <c r="E47" s="14">
         <v>6</v>
       </c>
-      <c r="F47" s="27"/>
-      <c r="G47" s="28"/>
-      <c r="H47" s="24"/>
+      <c r="F47" s="34"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="43"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A48" s="26">
+      <c r="A48" s="33">
         <v>46296</v>
       </c>
-      <c r="B48" s="26" t="s">
+      <c r="B48" s="33" t="s">
         <v>80</v>
       </c>
       <c r="C48" s="14" t="s">
@@ -2006,17 +2006,17 @@
         <v>2</v>
       </c>
       <c r="E48" s="13"/>
-      <c r="F48" s="27" t="s">
+      <c r="F48" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G48" s="28">
-        <v>6</v>
-      </c>
-      <c r="H48" s="24"/>
+      <c r="G48" s="35">
+        <v>6</v>
+      </c>
+      <c r="H48" s="43"/>
     </row>
     <row r="49" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A49" s="26"/>
-      <c r="B49" s="26"/>
+      <c r="A49" s="33"/>
+      <c r="B49" s="33"/>
       <c r="C49" s="14" t="s">
         <v>82</v>
       </c>
@@ -2024,13 +2024,13 @@
         <v>2</v>
       </c>
       <c r="E49" s="13"/>
-      <c r="F49" s="27"/>
-      <c r="G49" s="28"/>
-      <c r="H49" s="24"/>
+      <c r="F49" s="34"/>
+      <c r="G49" s="35"/>
+      <c r="H49" s="43"/>
     </row>
     <row r="50" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A50" s="26"/>
-      <c r="B50" s="26"/>
+      <c r="A50" s="33"/>
+      <c r="B50" s="33"/>
       <c r="C50" s="14" t="s">
         <v>83</v>
       </c>
@@ -2040,15 +2040,15 @@
       <c r="E50" s="14">
         <v>6</v>
       </c>
-      <c r="F50" s="27"/>
-      <c r="G50" s="28"/>
-      <c r="H50" s="24"/>
+      <c r="F50" s="34"/>
+      <c r="G50" s="35"/>
+      <c r="H50" s="43"/>
     </row>
     <row r="51" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A51" s="26">
+      <c r="A51" s="33">
         <v>46297</v>
       </c>
-      <c r="B51" s="26" t="s">
+      <c r="B51" s="33" t="s">
         <v>84</v>
       </c>
       <c r="C51" s="14" t="s">
@@ -2058,17 +2058,17 @@
         <v>2</v>
       </c>
       <c r="E51" s="13"/>
-      <c r="F51" s="27" t="s">
+      <c r="F51" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G51" s="28">
-        <v>6</v>
-      </c>
-      <c r="H51" s="24"/>
+      <c r="G51" s="35">
+        <v>6</v>
+      </c>
+      <c r="H51" s="43"/>
     </row>
     <row r="52" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A52" s="26"/>
-      <c r="B52" s="26"/>
+      <c r="A52" s="33"/>
+      <c r="B52" s="33"/>
       <c r="C52" s="14" t="s">
         <v>86</v>
       </c>
@@ -2076,13 +2076,13 @@
         <v>2</v>
       </c>
       <c r="E52" s="13"/>
-      <c r="F52" s="27"/>
-      <c r="G52" s="28"/>
-      <c r="H52" s="24"/>
+      <c r="F52" s="34"/>
+      <c r="G52" s="35"/>
+      <c r="H52" s="43"/>
     </row>
     <row r="53" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A53" s="26"/>
-      <c r="B53" s="26"/>
+      <c r="A53" s="33"/>
+      <c r="B53" s="33"/>
       <c r="C53" s="14" t="s">
         <v>87</v>
       </c>
@@ -2092,15 +2092,15 @@
       <c r="E53" s="14">
         <v>6</v>
       </c>
-      <c r="F53" s="27"/>
-      <c r="G53" s="28"/>
-      <c r="H53" s="24"/>
+      <c r="F53" s="34"/>
+      <c r="G53" s="35"/>
+      <c r="H53" s="43"/>
     </row>
     <row r="54" spans="1:8" ht="30.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A54" s="26">
+      <c r="A54" s="33">
         <v>46300</v>
       </c>
-      <c r="B54" s="26" t="s">
+      <c r="B54" s="33" t="s">
         <v>88</v>
       </c>
       <c r="C54" s="14" t="s">
@@ -2110,17 +2110,17 @@
         <v>2</v>
       </c>
       <c r="E54" s="13"/>
-      <c r="F54" s="27" t="s">
+      <c r="F54" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G54" s="28">
-        <v>6</v>
-      </c>
-      <c r="H54" s="24"/>
+      <c r="G54" s="35">
+        <v>6</v>
+      </c>
+      <c r="H54" s="43"/>
     </row>
     <row r="55" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A55" s="26"/>
-      <c r="B55" s="26"/>
+      <c r="A55" s="33"/>
+      <c r="B55" s="33"/>
       <c r="C55" s="14" t="s">
         <v>90</v>
       </c>
@@ -2128,13 +2128,13 @@
         <v>2</v>
       </c>
       <c r="E55" s="13"/>
-      <c r="F55" s="27"/>
-      <c r="G55" s="28"/>
-      <c r="H55" s="24"/>
+      <c r="F55" s="34"/>
+      <c r="G55" s="35"/>
+      <c r="H55" s="43"/>
     </row>
     <row r="56" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A56" s="26"/>
-      <c r="B56" s="26"/>
+      <c r="A56" s="33"/>
+      <c r="B56" s="33"/>
       <c r="C56" s="14" t="s">
         <v>91</v>
       </c>
@@ -2144,15 +2144,15 @@
       <c r="E56" s="14">
         <v>6</v>
       </c>
-      <c r="F56" s="27"/>
-      <c r="G56" s="28"/>
-      <c r="H56" s="24"/>
+      <c r="F56" s="34"/>
+      <c r="G56" s="35"/>
+      <c r="H56" s="43"/>
     </row>
     <row r="57" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A57" s="26">
+      <c r="A57" s="33">
         <v>46301</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="B57" s="33" t="s">
         <v>92</v>
       </c>
       <c r="C57" s="14" t="s">
@@ -2162,17 +2162,17 @@
         <v>2</v>
       </c>
       <c r="E57" s="13"/>
-      <c r="F57" s="27" t="s">
+      <c r="F57" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G57" s="28">
-        <v>6</v>
-      </c>
-      <c r="H57" s="24"/>
+      <c r="G57" s="35">
+        <v>6</v>
+      </c>
+      <c r="H57" s="43"/>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="26"/>
-      <c r="B58" s="26"/>
+      <c r="A58" s="33"/>
+      <c r="B58" s="33"/>
       <c r="C58" s="14" t="s">
         <v>94</v>
       </c>
@@ -2180,13 +2180,13 @@
         <v>2</v>
       </c>
       <c r="E58" s="13"/>
-      <c r="F58" s="27"/>
-      <c r="G58" s="28"/>
-      <c r="H58" s="24"/>
+      <c r="F58" s="34"/>
+      <c r="G58" s="35"/>
+      <c r="H58" s="43"/>
     </row>
     <row r="59" spans="1:8" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="26"/>
-      <c r="B59" s="26"/>
+      <c r="A59" s="33"/>
+      <c r="B59" s="33"/>
       <c r="C59" s="14" t="s">
         <v>95</v>
       </c>
@@ -2196,15 +2196,15 @@
       <c r="E59" s="14">
         <v>6</v>
       </c>
-      <c r="F59" s="27"/>
-      <c r="G59" s="28"/>
-      <c r="H59" s="24"/>
+      <c r="F59" s="34"/>
+      <c r="G59" s="35"/>
+      <c r="H59" s="43"/>
     </row>
     <row r="60" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A60" s="26">
+      <c r="A60" s="33">
         <v>46302</v>
       </c>
-      <c r="B60" s="26" t="s">
+      <c r="B60" s="33" t="s">
         <v>96</v>
       </c>
       <c r="C60" s="14" t="s">
@@ -2214,17 +2214,17 @@
         <v>2</v>
       </c>
       <c r="E60" s="13"/>
-      <c r="F60" s="27" t="s">
+      <c r="F60" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G60" s="28">
-        <v>6</v>
-      </c>
-      <c r="H60" s="24"/>
+      <c r="G60" s="35">
+        <v>6</v>
+      </c>
+      <c r="H60" s="43"/>
     </row>
     <row r="61" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A61" s="26"/>
-      <c r="B61" s="26"/>
+      <c r="A61" s="33"/>
+      <c r="B61" s="33"/>
       <c r="C61" s="14" t="s">
         <v>98</v>
       </c>
@@ -2232,13 +2232,13 @@
         <v>2</v>
       </c>
       <c r="E61" s="13"/>
-      <c r="F61" s="27"/>
-      <c r="G61" s="28"/>
-      <c r="H61" s="24"/>
+      <c r="F61" s="34"/>
+      <c r="G61" s="35"/>
+      <c r="H61" s="43"/>
     </row>
     <row r="62" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A62" s="26"/>
-      <c r="B62" s="26"/>
+      <c r="A62" s="33"/>
+      <c r="B62" s="33"/>
       <c r="C62" s="14" t="s">
         <v>99</v>
       </c>
@@ -2248,15 +2248,15 @@
       <c r="E62" s="14">
         <v>6</v>
       </c>
-      <c r="F62" s="27"/>
-      <c r="G62" s="28"/>
-      <c r="H62" s="24"/>
+      <c r="F62" s="34"/>
+      <c r="G62" s="35"/>
+      <c r="H62" s="43"/>
     </row>
     <row r="63" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A63" s="26">
+      <c r="A63" s="33">
         <v>46303</v>
       </c>
-      <c r="B63" s="26" t="s">
+      <c r="B63" s="33" t="s">
         <v>100</v>
       </c>
       <c r="C63" s="14" t="s">
@@ -2266,17 +2266,17 @@
         <v>2</v>
       </c>
       <c r="E63" s="13"/>
-      <c r="F63" s="27" t="s">
+      <c r="F63" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G63" s="28">
-        <v>6</v>
-      </c>
-      <c r="H63" s="24"/>
+      <c r="G63" s="35">
+        <v>6</v>
+      </c>
+      <c r="H63" s="43"/>
     </row>
     <row r="64" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A64" s="26"/>
-      <c r="B64" s="26"/>
+      <c r="A64" s="33"/>
+      <c r="B64" s="33"/>
       <c r="C64" s="14" t="s">
         <v>102</v>
       </c>
@@ -2284,13 +2284,13 @@
         <v>2</v>
       </c>
       <c r="E64" s="13"/>
-      <c r="F64" s="27"/>
-      <c r="G64" s="28"/>
-      <c r="H64" s="24"/>
+      <c r="F64" s="34"/>
+      <c r="G64" s="35"/>
+      <c r="H64" s="43"/>
     </row>
     <row r="65" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A65" s="26"/>
-      <c r="B65" s="26"/>
+      <c r="A65" s="33"/>
+      <c r="B65" s="33"/>
       <c r="C65" s="14" t="s">
         <v>173</v>
       </c>
@@ -2300,15 +2300,15 @@
       <c r="E65" s="14">
         <v>6</v>
       </c>
-      <c r="F65" s="27"/>
-      <c r="G65" s="28"/>
-      <c r="H65" s="24"/>
+      <c r="F65" s="34"/>
+      <c r="G65" s="35"/>
+      <c r="H65" s="43"/>
     </row>
     <row r="66" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="26">
+      <c r="A66" s="33">
         <v>46307</v>
       </c>
-      <c r="B66" s="26" t="s">
+      <c r="B66" s="33" t="s">
         <v>103</v>
       </c>
       <c r="C66" s="14" t="s">
@@ -2318,17 +2318,17 @@
         <v>2</v>
       </c>
       <c r="E66" s="13"/>
-      <c r="F66" s="27" t="s">
+      <c r="F66" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G66" s="28">
-        <v>6</v>
-      </c>
-      <c r="H66" s="24"/>
+      <c r="G66" s="35">
+        <v>6</v>
+      </c>
+      <c r="H66" s="43"/>
     </row>
     <row r="67" spans="1:8" ht="32.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A67" s="26"/>
-      <c r="B67" s="26"/>
+      <c r="A67" s="33"/>
+      <c r="B67" s="33"/>
       <c r="C67" s="14" t="s">
         <v>106</v>
       </c>
@@ -2336,13 +2336,13 @@
         <v>2</v>
       </c>
       <c r="E67" s="14"/>
-      <c r="F67" s="27"/>
-      <c r="G67" s="28"/>
-      <c r="H67" s="24"/>
+      <c r="F67" s="34"/>
+      <c r="G67" s="35"/>
+      <c r="H67" s="43"/>
     </row>
     <row r="68" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A68" s="26"/>
-      <c r="B68" s="26"/>
+      <c r="A68" s="33"/>
+      <c r="B68" s="33"/>
       <c r="C68" s="14" t="s">
         <v>107</v>
       </c>
@@ -2352,15 +2352,15 @@
       <c r="E68" s="14">
         <v>6</v>
       </c>
-      <c r="F68" s="27"/>
-      <c r="G68" s="28"/>
-      <c r="H68" s="24"/>
+      <c r="F68" s="34"/>
+      <c r="G68" s="35"/>
+      <c r="H68" s="43"/>
     </row>
     <row r="69" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A69" s="26">
+      <c r="A69" s="33">
         <v>46308</v>
       </c>
-      <c r="B69" s="28" t="s">
+      <c r="B69" s="35" t="s">
         <v>104</v>
       </c>
       <c r="C69" s="14" t="s">
@@ -2370,17 +2370,17 @@
         <v>2</v>
       </c>
       <c r="E69" s="14"/>
-      <c r="F69" s="27" t="s">
+      <c r="F69" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G69" s="28">
-        <v>6</v>
-      </c>
-      <c r="H69" s="24"/>
+      <c r="G69" s="35">
+        <v>6</v>
+      </c>
+      <c r="H69" s="43"/>
     </row>
     <row r="70" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A70" s="26"/>
-      <c r="B70" s="28"/>
+      <c r="A70" s="33"/>
+      <c r="B70" s="35"/>
       <c r="C70" s="14" t="s">
         <v>108</v>
       </c>
@@ -2388,13 +2388,13 @@
         <v>2</v>
       </c>
       <c r="E70" s="14"/>
-      <c r="F70" s="27"/>
-      <c r="G70" s="28"/>
-      <c r="H70" s="24"/>
+      <c r="F70" s="34"/>
+      <c r="G70" s="35"/>
+      <c r="H70" s="43"/>
     </row>
     <row r="71" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A71" s="26"/>
-      <c r="B71" s="28"/>
+      <c r="A71" s="33"/>
+      <c r="B71" s="35"/>
       <c r="C71" s="14" t="s">
         <v>143</v>
       </c>
@@ -2404,15 +2404,15 @@
       <c r="E71" s="14">
         <v>6</v>
       </c>
-      <c r="F71" s="27"/>
-      <c r="G71" s="28"/>
-      <c r="H71" s="24"/>
+      <c r="F71" s="34"/>
+      <c r="G71" s="35"/>
+      <c r="H71" s="43"/>
     </row>
     <row r="72" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="26">
+      <c r="A72" s="33">
         <v>46309</v>
       </c>
-      <c r="B72" s="28" t="s">
+      <c r="B72" s="35" t="s">
         <v>109</v>
       </c>
       <c r="C72" s="14" t="s">
@@ -2422,17 +2422,17 @@
         <v>2</v>
       </c>
       <c r="E72" s="14"/>
-      <c r="F72" s="27" t="s">
+      <c r="F72" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G72" s="28">
-        <v>6</v>
-      </c>
-      <c r="H72" s="24"/>
+      <c r="G72" s="35">
+        <v>6</v>
+      </c>
+      <c r="H72" s="43"/>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A73" s="26"/>
-      <c r="B73" s="28"/>
+      <c r="A73" s="33"/>
+      <c r="B73" s="35"/>
       <c r="C73" s="14" t="s">
         <v>110</v>
       </c>
@@ -2440,13 +2440,13 @@
         <v>2</v>
       </c>
       <c r="E73" s="14"/>
-      <c r="F73" s="27"/>
-      <c r="G73" s="28"/>
-      <c r="H73" s="24"/>
+      <c r="F73" s="34"/>
+      <c r="G73" s="35"/>
+      <c r="H73" s="43"/>
     </row>
     <row r="74" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A74" s="26"/>
-      <c r="B74" s="28"/>
+      <c r="A74" s="33"/>
+      <c r="B74" s="35"/>
       <c r="C74" s="14" t="s">
         <v>111</v>
       </c>
@@ -2456,15 +2456,15 @@
       <c r="E74" s="14">
         <v>6</v>
       </c>
-      <c r="F74" s="27"/>
-      <c r="G74" s="28"/>
-      <c r="H74" s="24"/>
+      <c r="F74" s="34"/>
+      <c r="G74" s="35"/>
+      <c r="H74" s="43"/>
     </row>
     <row r="75" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A75" s="26">
+      <c r="A75" s="33">
         <v>46310</v>
       </c>
-      <c r="B75" s="28" t="s">
+      <c r="B75" s="35" t="s">
         <v>49</v>
       </c>
       <c r="C75" s="14" t="s">
@@ -2474,17 +2474,17 @@
         <v>2</v>
       </c>
       <c r="E75" s="14"/>
-      <c r="F75" s="27" t="s">
+      <c r="F75" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G75" s="28">
-        <v>6</v>
-      </c>
-      <c r="H75" s="24"/>
+      <c r="G75" s="35">
+        <v>6</v>
+      </c>
+      <c r="H75" s="43"/>
     </row>
     <row r="76" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A76" s="26"/>
-      <c r="B76" s="28"/>
+      <c r="A76" s="33"/>
+      <c r="B76" s="35"/>
       <c r="C76" s="14" t="s">
         <v>113</v>
       </c>
@@ -2492,13 +2492,13 @@
         <v>2</v>
       </c>
       <c r="E76" s="14"/>
-      <c r="F76" s="27"/>
-      <c r="G76" s="28"/>
-      <c r="H76" s="24"/>
+      <c r="F76" s="34"/>
+      <c r="G76" s="35"/>
+      <c r="H76" s="43"/>
     </row>
     <row r="77" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A77" s="26"/>
-      <c r="B77" s="28"/>
+      <c r="A77" s="33"/>
+      <c r="B77" s="35"/>
       <c r="C77" s="14" t="s">
         <v>114</v>
       </c>
@@ -2508,15 +2508,15 @@
       <c r="E77" s="14">
         <v>6</v>
       </c>
-      <c r="F77" s="27"/>
-      <c r="G77" s="28"/>
-      <c r="H77" s="24"/>
+      <c r="F77" s="34"/>
+      <c r="G77" s="35"/>
+      <c r="H77" s="43"/>
     </row>
     <row r="78" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A78" s="26">
+      <c r="A78" s="33">
         <v>46311</v>
       </c>
-      <c r="B78" s="26" t="s">
+      <c r="B78" s="33" t="s">
         <v>49</v>
       </c>
       <c r="C78" s="14" t="s">
@@ -2526,17 +2526,17 @@
         <v>2</v>
       </c>
       <c r="E78" s="14"/>
-      <c r="F78" s="27" t="s">
+      <c r="F78" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G78" s="28">
-        <v>6</v>
-      </c>
-      <c r="H78" s="24"/>
+      <c r="G78" s="35">
+        <v>6</v>
+      </c>
+      <c r="H78" s="43"/>
     </row>
     <row r="79" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A79" s="26"/>
-      <c r="B79" s="26"/>
+      <c r="A79" s="33"/>
+      <c r="B79" s="33"/>
       <c r="C79" s="14" t="s">
         <v>116</v>
       </c>
@@ -2544,13 +2544,13 @@
         <v>2</v>
       </c>
       <c r="E79" s="14"/>
-      <c r="F79" s="27"/>
-      <c r="G79" s="28"/>
-      <c r="H79" s="24"/>
+      <c r="F79" s="34"/>
+      <c r="G79" s="35"/>
+      <c r="H79" s="43"/>
     </row>
     <row r="80" spans="1:8" ht="33.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A80" s="26"/>
-      <c r="B80" s="26"/>
+      <c r="A80" s="33"/>
+      <c r="B80" s="33"/>
       <c r="C80" s="14" t="s">
         <v>117</v>
       </c>
@@ -2560,15 +2560,15 @@
       <c r="E80" s="14">
         <v>6</v>
       </c>
-      <c r="F80" s="27"/>
-      <c r="G80" s="28"/>
-      <c r="H80" s="24"/>
+      <c r="F80" s="34"/>
+      <c r="G80" s="35"/>
+      <c r="H80" s="43"/>
     </row>
     <row r="81" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A81" s="26">
+      <c r="A81" s="33">
         <v>46314</v>
       </c>
-      <c r="B81" s="26" t="s">
+      <c r="B81" s="33" t="s">
         <v>118</v>
       </c>
       <c r="C81" s="20" t="s">
@@ -2578,17 +2578,17 @@
         <v>2</v>
       </c>
       <c r="E81" s="14"/>
-      <c r="F81" s="27" t="s">
+      <c r="F81" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G81" s="28">
-        <v>6</v>
-      </c>
-      <c r="H81" s="25"/>
+      <c r="G81" s="35">
+        <v>6</v>
+      </c>
+      <c r="H81" s="44"/>
     </row>
     <row r="82" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A82" s="26"/>
-      <c r="B82" s="26"/>
+      <c r="A82" s="33"/>
+      <c r="B82" s="33"/>
       <c r="C82" s="20" t="s">
         <v>120</v>
       </c>
@@ -2596,13 +2596,13 @@
         <v>2</v>
       </c>
       <c r="E82" s="14"/>
-      <c r="F82" s="27"/>
-      <c r="G82" s="28"/>
-      <c r="H82" s="25"/>
+      <c r="F82" s="34"/>
+      <c r="G82" s="35"/>
+      <c r="H82" s="44"/>
     </row>
     <row r="83" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A83" s="26"/>
-      <c r="B83" s="26"/>
+      <c r="A83" s="33"/>
+      <c r="B83" s="33"/>
       <c r="C83" s="14" t="s">
         <v>121</v>
       </c>
@@ -2612,15 +2612,15 @@
       <c r="E83" s="14">
         <v>6</v>
       </c>
-      <c r="F83" s="27"/>
-      <c r="G83" s="28"/>
-      <c r="H83" s="25"/>
+      <c r="F83" s="34"/>
+      <c r="G83" s="35"/>
+      <c r="H83" s="44"/>
     </row>
     <row r="84" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A84" s="26">
+      <c r="A84" s="33">
         <v>46315</v>
       </c>
-      <c r="B84" s="26" t="s">
+      <c r="B84" s="33" t="s">
         <v>50</v>
       </c>
       <c r="C84" s="14" t="s">
@@ -2630,17 +2630,17 @@
         <v>2</v>
       </c>
       <c r="E84" s="14"/>
-      <c r="F84" s="27" t="s">
+      <c r="F84" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G84" s="28">
-        <v>6</v>
-      </c>
-      <c r="H84" s="24"/>
+      <c r="G84" s="35">
+        <v>6</v>
+      </c>
+      <c r="H84" s="43"/>
     </row>
     <row r="85" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A85" s="26"/>
-      <c r="B85" s="26"/>
+      <c r="A85" s="33"/>
+      <c r="B85" s="33"/>
       <c r="C85" s="14" t="s">
         <v>123</v>
       </c>
@@ -2648,13 +2648,13 @@
         <v>2</v>
       </c>
       <c r="E85" s="14"/>
-      <c r="F85" s="27"/>
-      <c r="G85" s="28"/>
-      <c r="H85" s="24"/>
+      <c r="F85" s="34"/>
+      <c r="G85" s="35"/>
+      <c r="H85" s="43"/>
     </row>
     <row r="86" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A86" s="26"/>
-      <c r="B86" s="26"/>
+      <c r="A86" s="33"/>
+      <c r="B86" s="33"/>
       <c r="C86" s="20" t="s">
         <v>124</v>
       </c>
@@ -2664,15 +2664,15 @@
       <c r="E86" s="14">
         <v>6</v>
       </c>
-      <c r="F86" s="27"/>
-      <c r="G86" s="28"/>
-      <c r="H86" s="24"/>
+      <c r="F86" s="34"/>
+      <c r="G86" s="35"/>
+      <c r="H86" s="43"/>
     </row>
     <row r="87" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A87" s="26">
+      <c r="A87" s="33">
         <v>46316</v>
       </c>
-      <c r="B87" s="26" t="s">
+      <c r="B87" s="33" t="s">
         <v>50</v>
       </c>
       <c r="C87" s="14" t="s">
@@ -2682,17 +2682,17 @@
         <v>2</v>
       </c>
       <c r="E87" s="14"/>
-      <c r="F87" s="27" t="s">
+      <c r="F87" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G87" s="28">
-        <v>6</v>
-      </c>
-      <c r="H87" s="24"/>
+      <c r="G87" s="35">
+        <v>6</v>
+      </c>
+      <c r="H87" s="43"/>
     </row>
     <row r="88" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A88" s="26"/>
-      <c r="B88" s="26"/>
+      <c r="A88" s="33"/>
+      <c r="B88" s="33"/>
       <c r="C88" s="14" t="s">
         <v>126</v>
       </c>
@@ -2700,13 +2700,13 @@
         <v>2</v>
       </c>
       <c r="E88" s="13"/>
-      <c r="F88" s="27"/>
-      <c r="G88" s="28"/>
-      <c r="H88" s="24"/>
+      <c r="F88" s="34"/>
+      <c r="G88" s="35"/>
+      <c r="H88" s="43"/>
     </row>
     <row r="89" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A89" s="26"/>
-      <c r="B89" s="26"/>
+      <c r="A89" s="33"/>
+      <c r="B89" s="33"/>
       <c r="C89" s="14" t="s">
         <v>127</v>
       </c>
@@ -2716,15 +2716,15 @@
       <c r="E89" s="14">
         <v>6</v>
       </c>
-      <c r="F89" s="27"/>
-      <c r="G89" s="28"/>
-      <c r="H89" s="24"/>
+      <c r="F89" s="34"/>
+      <c r="G89" s="35"/>
+      <c r="H89" s="43"/>
     </row>
     <row r="90" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A90" s="26">
+      <c r="A90" s="33">
         <v>46317</v>
       </c>
-      <c r="B90" s="28" t="s">
+      <c r="B90" s="35" t="s">
         <v>130</v>
       </c>
       <c r="C90" s="14" t="s">
@@ -2734,17 +2734,17 @@
         <v>2</v>
       </c>
       <c r="E90" s="13"/>
-      <c r="F90" s="27" t="s">
+      <c r="F90" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G90" s="28">
-        <v>6</v>
-      </c>
-      <c r="H90" s="24"/>
+      <c r="G90" s="35">
+        <v>6</v>
+      </c>
+      <c r="H90" s="43"/>
     </row>
     <row r="91" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A91" s="26"/>
-      <c r="B91" s="28"/>
+      <c r="A91" s="33"/>
+      <c r="B91" s="35"/>
       <c r="C91" s="14" t="s">
         <v>120</v>
       </c>
@@ -2752,13 +2752,13 @@
         <v>2</v>
       </c>
       <c r="E91" s="13"/>
-      <c r="F91" s="27"/>
-      <c r="G91" s="28"/>
-      <c r="H91" s="24"/>
+      <c r="F91" s="34"/>
+      <c r="G91" s="35"/>
+      <c r="H91" s="43"/>
     </row>
     <row r="92" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A92" s="26"/>
-      <c r="B92" s="28"/>
+      <c r="A92" s="33"/>
+      <c r="B92" s="35"/>
       <c r="C92" s="14" t="s">
         <v>129</v>
       </c>
@@ -2768,15 +2768,15 @@
       <c r="E92" s="14">
         <v>6</v>
       </c>
-      <c r="F92" s="27"/>
-      <c r="G92" s="28"/>
-      <c r="H92" s="24"/>
+      <c r="F92" s="34"/>
+      <c r="G92" s="35"/>
+      <c r="H92" s="43"/>
     </row>
     <row r="93" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A93" s="26">
+      <c r="A93" s="33">
         <v>46318</v>
       </c>
-      <c r="B93" s="28" t="s">
+      <c r="B93" s="35" t="s">
         <v>51</v>
       </c>
       <c r="C93" s="20" t="s">
@@ -2786,17 +2786,17 @@
         <v>2</v>
       </c>
       <c r="E93" s="13"/>
-      <c r="F93" s="27" t="s">
+      <c r="F93" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G93" s="28">
-        <v>6</v>
-      </c>
-      <c r="H93" s="24"/>
+      <c r="G93" s="35">
+        <v>6</v>
+      </c>
+      <c r="H93" s="43"/>
     </row>
     <row r="94" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A94" s="26"/>
-      <c r="B94" s="28"/>
+      <c r="A94" s="33"/>
+      <c r="B94" s="35"/>
       <c r="C94" s="20" t="s">
         <v>132</v>
       </c>
@@ -2804,13 +2804,13 @@
         <v>2</v>
       </c>
       <c r="E94" s="13"/>
-      <c r="F94" s="27"/>
-      <c r="G94" s="28"/>
-      <c r="H94" s="24"/>
+      <c r="F94" s="34"/>
+      <c r="G94" s="35"/>
+      <c r="H94" s="43"/>
     </row>
     <row r="95" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A95" s="26"/>
-      <c r="B95" s="28"/>
+      <c r="A95" s="33"/>
+      <c r="B95" s="35"/>
       <c r="C95" s="14" t="s">
         <v>133</v>
       </c>
@@ -2820,15 +2820,15 @@
       <c r="E95" s="14">
         <v>6</v>
       </c>
-      <c r="F95" s="27"/>
-      <c r="G95" s="28"/>
-      <c r="H95" s="24"/>
+      <c r="F95" s="34"/>
+      <c r="G95" s="35"/>
+      <c r="H95" s="43"/>
     </row>
     <row r="96" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A96" s="26">
+      <c r="A96" s="33">
         <v>46321</v>
       </c>
-      <c r="B96" s="28" t="s">
+      <c r="B96" s="35" t="s">
         <v>51</v>
       </c>
       <c r="C96" s="14" t="s">
@@ -2838,17 +2838,17 @@
         <v>2</v>
       </c>
       <c r="E96" s="14"/>
-      <c r="F96" s="27" t="s">
+      <c r="F96" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G96" s="28">
-        <v>6</v>
-      </c>
-      <c r="H96" s="24"/>
+      <c r="G96" s="35">
+        <v>6</v>
+      </c>
+      <c r="H96" s="43"/>
     </row>
     <row r="97" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A97" s="26"/>
-      <c r="B97" s="28"/>
+      <c r="A97" s="33"/>
+      <c r="B97" s="35"/>
       <c r="C97" s="20" t="s">
         <v>135</v>
       </c>
@@ -2856,13 +2856,13 @@
         <v>2</v>
       </c>
       <c r="E97" s="13"/>
-      <c r="F97" s="27"/>
-      <c r="G97" s="28"/>
-      <c r="H97" s="24"/>
+      <c r="F97" s="34"/>
+      <c r="G97" s="35"/>
+      <c r="H97" s="43"/>
     </row>
     <row r="98" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A98" s="26"/>
-      <c r="B98" s="28"/>
+      <c r="A98" s="33"/>
+      <c r="B98" s="35"/>
       <c r="C98" s="14" t="s">
         <v>136</v>
       </c>
@@ -2872,15 +2872,15 @@
       <c r="E98" s="14">
         <v>6</v>
       </c>
-      <c r="F98" s="27"/>
-      <c r="G98" s="28"/>
-      <c r="H98" s="24"/>
+      <c r="F98" s="34"/>
+      <c r="G98" s="35"/>
+      <c r="H98" s="43"/>
     </row>
     <row r="99" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A99" s="26">
+      <c r="A99" s="33">
         <v>46322</v>
       </c>
-      <c r="B99" s="28" t="s">
+      <c r="B99" s="35" t="s">
         <v>137</v>
       </c>
       <c r="C99" s="14" t="s">
@@ -2890,17 +2890,17 @@
         <v>2</v>
       </c>
       <c r="E99" s="13"/>
-      <c r="F99" s="27" t="s">
+      <c r="F99" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G99" s="28">
-        <v>6</v>
-      </c>
-      <c r="H99" s="24"/>
+      <c r="G99" s="35">
+        <v>6</v>
+      </c>
+      <c r="H99" s="43"/>
     </row>
     <row r="100" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A100" s="26"/>
-      <c r="B100" s="28"/>
+      <c r="A100" s="33"/>
+      <c r="B100" s="35"/>
       <c r="C100" s="14" t="s">
         <v>120</v>
       </c>
@@ -2908,13 +2908,13 @@
         <v>2</v>
       </c>
       <c r="E100" s="13"/>
-      <c r="F100" s="27"/>
-      <c r="G100" s="28"/>
-      <c r="H100" s="24"/>
+      <c r="F100" s="34"/>
+      <c r="G100" s="35"/>
+      <c r="H100" s="43"/>
     </row>
     <row r="101" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A101" s="26"/>
-      <c r="B101" s="28"/>
+      <c r="A101" s="33"/>
+      <c r="B101" s="35"/>
       <c r="C101" s="14" t="s">
         <v>139</v>
       </c>
@@ -2924,15 +2924,15 @@
       <c r="E101" s="14">
         <v>6</v>
       </c>
-      <c r="F101" s="27"/>
-      <c r="G101" s="28"/>
-      <c r="H101" s="24"/>
+      <c r="F101" s="34"/>
+      <c r="G101" s="35"/>
+      <c r="H101" s="43"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A102" s="26">
+      <c r="A102" s="33">
         <v>46323</v>
       </c>
-      <c r="B102" s="28" t="s">
+      <c r="B102" s="35" t="s">
         <v>140</v>
       </c>
       <c r="C102" s="14" t="s">
@@ -2942,17 +2942,17 @@
         <v>2</v>
       </c>
       <c r="E102" s="14"/>
-      <c r="F102" s="27" t="s">
+      <c r="F102" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G102" s="28">
-        <v>6</v>
-      </c>
-      <c r="H102" s="24"/>
+      <c r="G102" s="35">
+        <v>6</v>
+      </c>
+      <c r="H102" s="43"/>
     </row>
     <row r="103" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A103" s="26"/>
-      <c r="B103" s="28"/>
+      <c r="A103" s="33"/>
+      <c r="B103" s="35"/>
       <c r="C103" s="20" t="s">
         <v>142</v>
       </c>
@@ -2960,13 +2960,13 @@
         <v>2</v>
       </c>
       <c r="E103" s="13"/>
-      <c r="F103" s="27"/>
-      <c r="G103" s="28"/>
-      <c r="H103" s="24"/>
+      <c r="F103" s="34"/>
+      <c r="G103" s="35"/>
+      <c r="H103" s="43"/>
     </row>
     <row r="104" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A104" s="26"/>
-      <c r="B104" s="28"/>
+      <c r="A104" s="33"/>
+      <c r="B104" s="35"/>
       <c r="C104" s="14" t="s">
         <v>144</v>
       </c>
@@ -2976,15 +2976,15 @@
       <c r="E104" s="14">
         <v>6</v>
       </c>
-      <c r="F104" s="27"/>
-      <c r="G104" s="28"/>
-      <c r="H104" s="24"/>
+      <c r="F104" s="34"/>
+      <c r="G104" s="35"/>
+      <c r="H104" s="43"/>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A105" s="26">
+      <c r="A105" s="33">
         <v>46324</v>
       </c>
-      <c r="B105" s="27" t="s">
+      <c r="B105" s="34" t="s">
         <v>145</v>
       </c>
       <c r="C105" s="14" t="s">
@@ -2994,17 +2994,17 @@
         <v>2</v>
       </c>
       <c r="E105" s="13"/>
-      <c r="F105" s="27" t="s">
+      <c r="F105" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G105" s="28">
-        <v>6</v>
-      </c>
-      <c r="H105" s="24"/>
+      <c r="G105" s="35">
+        <v>6</v>
+      </c>
+      <c r="H105" s="43"/>
     </row>
     <row r="106" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A106" s="26"/>
-      <c r="B106" s="27"/>
+      <c r="A106" s="33"/>
+      <c r="B106" s="34"/>
       <c r="C106" s="14" t="s">
         <v>147</v>
       </c>
@@ -3012,13 +3012,13 @@
         <v>2</v>
       </c>
       <c r="E106" s="13"/>
-      <c r="F106" s="27"/>
-      <c r="G106" s="28"/>
-      <c r="H106" s="24"/>
+      <c r="F106" s="34"/>
+      <c r="G106" s="35"/>
+      <c r="H106" s="43"/>
     </row>
     <row r="107" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A107" s="26"/>
-      <c r="B107" s="27"/>
+      <c r="A107" s="33"/>
+      <c r="B107" s="34"/>
       <c r="C107" s="14" t="s">
         <v>148</v>
       </c>
@@ -3028,15 +3028,15 @@
       <c r="E107" s="14">
         <v>6</v>
       </c>
-      <c r="F107" s="27"/>
-      <c r="G107" s="28"/>
-      <c r="H107" s="24"/>
+      <c r="F107" s="34"/>
+      <c r="G107" s="35"/>
+      <c r="H107" s="43"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A108" s="26">
+      <c r="A108" s="33">
         <v>46325</v>
       </c>
-      <c r="B108" s="27" t="s">
+      <c r="B108" s="34" t="s">
         <v>149</v>
       </c>
       <c r="C108" s="14" t="s">
@@ -3046,17 +3046,17 @@
         <v>2</v>
       </c>
       <c r="E108" s="13"/>
-      <c r="F108" s="27" t="s">
+      <c r="F108" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G108" s="28">
-        <v>6</v>
-      </c>
-      <c r="H108" s="24"/>
+      <c r="G108" s="35">
+        <v>6</v>
+      </c>
+      <c r="H108" s="43"/>
     </row>
     <row r="109" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A109" s="26"/>
-      <c r="B109" s="27"/>
+      <c r="A109" s="33"/>
+      <c r="B109" s="34"/>
       <c r="C109" s="15" t="s">
         <v>151</v>
       </c>
@@ -3064,13 +3064,13 @@
         <v>2</v>
       </c>
       <c r="E109" s="13"/>
-      <c r="F109" s="27"/>
-      <c r="G109" s="28"/>
-      <c r="H109" s="24"/>
+      <c r="F109" s="34"/>
+      <c r="G109" s="35"/>
+      <c r="H109" s="43"/>
     </row>
     <row r="110" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A110" s="26"/>
-      <c r="B110" s="27"/>
+      <c r="A110" s="33"/>
+      <c r="B110" s="34"/>
       <c r="C110" s="14" t="s">
         <v>152</v>
       </c>
@@ -3080,15 +3080,15 @@
       <c r="E110" s="14">
         <v>6</v>
       </c>
-      <c r="F110" s="27"/>
-      <c r="G110" s="28"/>
-      <c r="H110" s="24"/>
+      <c r="F110" s="34"/>
+      <c r="G110" s="35"/>
+      <c r="H110" s="43"/>
     </row>
     <row r="111" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A111" s="26">
+      <c r="A111" s="33">
         <v>46330</v>
       </c>
-      <c r="B111" s="27" t="s">
+      <c r="B111" s="34" t="s">
         <v>153</v>
       </c>
       <c r="C111" s="14" t="s">
@@ -3098,17 +3098,17 @@
         <v>2</v>
       </c>
       <c r="E111" s="13"/>
-      <c r="F111" s="27" t="s">
+      <c r="F111" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G111" s="28">
-        <v>6</v>
-      </c>
-      <c r="H111" s="24"/>
+      <c r="G111" s="35">
+        <v>6</v>
+      </c>
+      <c r="H111" s="43"/>
     </row>
     <row r="112" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A112" s="26"/>
-      <c r="B112" s="27"/>
+      <c r="A112" s="33"/>
+      <c r="B112" s="34"/>
       <c r="C112" s="14" t="s">
         <v>155</v>
       </c>
@@ -3116,13 +3116,13 @@
         <v>2</v>
       </c>
       <c r="E112" s="13"/>
-      <c r="F112" s="27"/>
-      <c r="G112" s="28"/>
-      <c r="H112" s="24"/>
+      <c r="F112" s="34"/>
+      <c r="G112" s="35"/>
+      <c r="H112" s="43"/>
     </row>
     <row r="113" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A113" s="26"/>
-      <c r="B113" s="27"/>
+      <c r="A113" s="33"/>
+      <c r="B113" s="34"/>
       <c r="C113" s="14" t="s">
         <v>156</v>
       </c>
@@ -3132,15 +3132,15 @@
       <c r="E113" s="14">
         <v>6</v>
       </c>
-      <c r="F113" s="27"/>
-      <c r="G113" s="28"/>
-      <c r="H113" s="24"/>
+      <c r="F113" s="34"/>
+      <c r="G113" s="35"/>
+      <c r="H113" s="43"/>
     </row>
     <row r="114" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A114" s="26">
+      <c r="A114" s="33">
         <v>46331</v>
       </c>
-      <c r="B114" s="27" t="s">
+      <c r="B114" s="34" t="s">
         <v>157</v>
       </c>
       <c r="C114" s="14" t="s">
@@ -3150,17 +3150,17 @@
         <v>2</v>
       </c>
       <c r="E114" s="13"/>
-      <c r="F114" s="27" t="s">
+      <c r="F114" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G114" s="28">
-        <v>6</v>
-      </c>
-      <c r="H114" s="24"/>
+      <c r="G114" s="35">
+        <v>6</v>
+      </c>
+      <c r="H114" s="43"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A115" s="26"/>
-      <c r="B115" s="27"/>
+      <c r="A115" s="33"/>
+      <c r="B115" s="34"/>
       <c r="C115" s="14" t="s">
         <v>159</v>
       </c>
@@ -3168,13 +3168,13 @@
         <v>2</v>
       </c>
       <c r="E115" s="13"/>
-      <c r="F115" s="27"/>
-      <c r="G115" s="28"/>
-      <c r="H115" s="24"/>
+      <c r="F115" s="34"/>
+      <c r="G115" s="35"/>
+      <c r="H115" s="43"/>
     </row>
     <row r="116" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A116" s="26"/>
-      <c r="B116" s="27"/>
+      <c r="A116" s="33"/>
+      <c r="B116" s="34"/>
       <c r="C116" s="14" t="s">
         <v>160</v>
       </c>
@@ -3184,15 +3184,15 @@
       <c r="E116" s="14">
         <v>6</v>
       </c>
-      <c r="F116" s="27"/>
-      <c r="G116" s="28"/>
-      <c r="H116" s="24"/>
+      <c r="F116" s="34"/>
+      <c r="G116" s="35"/>
+      <c r="H116" s="43"/>
     </row>
     <row r="117" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A117" s="26">
+      <c r="A117" s="33">
         <v>46332</v>
       </c>
-      <c r="B117" s="27" t="s">
+      <c r="B117" s="34" t="s">
         <v>161</v>
       </c>
       <c r="C117" s="14" t="s">
@@ -3202,17 +3202,17 @@
         <v>2</v>
       </c>
       <c r="E117" s="13"/>
-      <c r="F117" s="27" t="s">
+      <c r="F117" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G117" s="28">
-        <v>6</v>
-      </c>
-      <c r="H117" s="24"/>
+      <c r="G117" s="35">
+        <v>6</v>
+      </c>
+      <c r="H117" s="43"/>
     </row>
     <row r="118" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A118" s="26"/>
-      <c r="B118" s="27"/>
+      <c r="A118" s="33"/>
+      <c r="B118" s="34"/>
       <c r="C118" s="14" t="s">
         <v>163</v>
       </c>
@@ -3220,13 +3220,13 @@
         <v>2</v>
       </c>
       <c r="E118" s="13"/>
-      <c r="F118" s="27"/>
-      <c r="G118" s="28"/>
-      <c r="H118" s="24"/>
+      <c r="F118" s="34"/>
+      <c r="G118" s="35"/>
+      <c r="H118" s="43"/>
     </row>
     <row r="119" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A119" s="26"/>
-      <c r="B119" s="27"/>
+      <c r="A119" s="33"/>
+      <c r="B119" s="34"/>
       <c r="C119" s="14" t="s">
         <v>176</v>
       </c>
@@ -3236,15 +3236,15 @@
       <c r="E119" s="14">
         <v>6</v>
       </c>
-      <c r="F119" s="27"/>
-      <c r="G119" s="28"/>
-      <c r="H119" s="24"/>
+      <c r="F119" s="34"/>
+      <c r="G119" s="35"/>
+      <c r="H119" s="43"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A120" s="39">
+      <c r="A120" s="36">
         <v>46335</v>
       </c>
-      <c r="B120" s="30" t="s">
+      <c r="B120" s="24" t="s">
         <v>164</v>
       </c>
       <c r="C120" s="22" t="s">
@@ -3254,17 +3254,17 @@
         <v>2</v>
       </c>
       <c r="E120" s="22"/>
-      <c r="F120" s="30" t="s">
+      <c r="F120" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G120" s="33">
-        <v>6</v>
-      </c>
-      <c r="H120" s="36"/>
+      <c r="G120" s="27">
+        <v>6</v>
+      </c>
+      <c r="H120" s="30"/>
     </row>
     <row r="121" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A121" s="40"/>
-      <c r="B121" s="31"/>
+      <c r="A121" s="37"/>
+      <c r="B121" s="25"/>
       <c r="C121" s="22" t="s">
         <v>166</v>
       </c>
@@ -3272,51 +3272,51 @@
         <v>2</v>
       </c>
       <c r="E121" s="22"/>
-      <c r="F121" s="31"/>
-      <c r="G121" s="34"/>
-      <c r="H121" s="37"/>
+      <c r="F121" s="25"/>
+      <c r="G121" s="28"/>
+      <c r="H121" s="31"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A122" s="40"/>
-      <c r="B122" s="31"/>
-      <c r="C122" s="30" t="s">
+      <c r="A122" s="37"/>
+      <c r="B122" s="25"/>
+      <c r="C122" s="24" t="s">
         <v>167</v>
       </c>
-      <c r="D122" s="42">
-        <v>2</v>
-      </c>
-      <c r="E122" s="42">
-        <v>6</v>
-      </c>
-      <c r="F122" s="31"/>
-      <c r="G122" s="34"/>
-      <c r="H122" s="37"/>
+      <c r="D122" s="39">
+        <v>2</v>
+      </c>
+      <c r="E122" s="39">
+        <v>6</v>
+      </c>
+      <c r="F122" s="25"/>
+      <c r="G122" s="28"/>
+      <c r="H122" s="31"/>
     </row>
     <row r="123" spans="1:8" ht="11.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A123" s="40"/>
-      <c r="B123" s="31"/>
-      <c r="C123" s="31"/>
-      <c r="D123" s="43"/>
-      <c r="E123" s="43"/>
-      <c r="F123" s="31"/>
-      <c r="G123" s="34"/>
-      <c r="H123" s="37"/>
+      <c r="A123" s="37"/>
+      <c r="B123" s="25"/>
+      <c r="C123" s="25"/>
+      <c r="D123" s="40"/>
+      <c r="E123" s="40"/>
+      <c r="F123" s="25"/>
+      <c r="G123" s="28"/>
+      <c r="H123" s="31"/>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A124" s="41"/>
-      <c r="B124" s="32"/>
-      <c r="C124" s="32"/>
-      <c r="D124" s="44"/>
-      <c r="E124" s="44"/>
-      <c r="F124" s="32"/>
-      <c r="G124" s="35"/>
-      <c r="H124" s="38"/>
+      <c r="A124" s="38"/>
+      <c r="B124" s="26"/>
+      <c r="C124" s="26"/>
+      <c r="D124" s="41"/>
+      <c r="E124" s="41"/>
+      <c r="F124" s="26"/>
+      <c r="G124" s="29"/>
+      <c r="H124" s="32"/>
     </row>
     <row r="125" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A125" s="26">
+      <c r="A125" s="33">
         <v>46336</v>
       </c>
-      <c r="B125" s="27" t="s">
+      <c r="B125" s="34" t="s">
         <v>168</v>
       </c>
       <c r="C125" s="14" t="s">
@@ -3326,17 +3326,17 @@
         <v>2</v>
       </c>
       <c r="E125" s="13"/>
-      <c r="F125" s="27" t="s">
+      <c r="F125" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G125" s="28">
-        <v>6</v>
-      </c>
-      <c r="H125" s="24"/>
+      <c r="G125" s="35">
+        <v>6</v>
+      </c>
+      <c r="H125" s="43"/>
     </row>
     <row r="126" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A126" s="26"/>
-      <c r="B126" s="27"/>
+      <c r="A126" s="33"/>
+      <c r="B126" s="34"/>
       <c r="C126" s="14" t="s">
         <v>169</v>
       </c>
@@ -3344,13 +3344,13 @@
         <v>2</v>
       </c>
       <c r="E126" s="13"/>
-      <c r="F126" s="27"/>
-      <c r="G126" s="28"/>
-      <c r="H126" s="24"/>
+      <c r="F126" s="34"/>
+      <c r="G126" s="35"/>
+      <c r="H126" s="43"/>
     </row>
     <row r="127" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A127" s="26"/>
-      <c r="B127" s="27"/>
+      <c r="A127" s="33"/>
+      <c r="B127" s="34"/>
       <c r="C127" s="14" t="s">
         <v>170</v>
       </c>
@@ -3360,15 +3360,15 @@
       <c r="E127" s="14">
         <v>6</v>
       </c>
-      <c r="F127" s="27"/>
-      <c r="G127" s="28"/>
-      <c r="H127" s="24"/>
+      <c r="F127" s="34"/>
+      <c r="G127" s="35"/>
+      <c r="H127" s="43"/>
     </row>
     <row r="128" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A128" s="26">
+      <c r="A128" s="33">
         <v>46337</v>
       </c>
-      <c r="B128" s="27" t="s">
+      <c r="B128" s="34" t="s">
         <v>52</v>
       </c>
       <c r="C128" s="14" t="s">
@@ -3378,17 +3378,17 @@
         <v>2</v>
       </c>
       <c r="E128" s="13"/>
-      <c r="F128" s="27" t="s">
+      <c r="F128" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="G128" s="28">
-        <v>6</v>
-      </c>
-      <c r="H128" s="24"/>
+      <c r="G128" s="35">
+        <v>6</v>
+      </c>
+      <c r="H128" s="43"/>
     </row>
     <row r="129" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A129" s="26"/>
-      <c r="B129" s="27"/>
+      <c r="A129" s="33"/>
+      <c r="B129" s="34"/>
       <c r="C129" s="14" t="s">
         <v>172</v>
       </c>
@@ -3396,13 +3396,13 @@
         <v>2</v>
       </c>
       <c r="E129" s="13"/>
-      <c r="F129" s="27"/>
-      <c r="G129" s="28"/>
-      <c r="H129" s="24"/>
+      <c r="F129" s="34"/>
+      <c r="G129" s="35"/>
+      <c r="H129" s="43"/>
     </row>
     <row r="130" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A130" s="26"/>
-      <c r="B130" s="27"/>
+      <c r="A130" s="33"/>
+      <c r="B130" s="34"/>
       <c r="C130" s="14" t="s">
         <v>53</v>
       </c>
@@ -3412,9 +3412,9 @@
       <c r="E130" s="14">
         <v>6</v>
       </c>
-      <c r="F130" s="27"/>
-      <c r="G130" s="28"/>
-      <c r="H130" s="24"/>
+      <c r="F130" s="34"/>
+      <c r="G130" s="35"/>
+      <c r="H130" s="43"/>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A131" s="11"/>
@@ -3527,6 +3527,186 @@
     </row>
   </sheetData>
   <mergeCells count="204">
+    <mergeCell ref="H90:H92"/>
+    <mergeCell ref="H93:H95"/>
+    <mergeCell ref="H96:H98"/>
+    <mergeCell ref="H128:H130"/>
+    <mergeCell ref="H99:H101"/>
+    <mergeCell ref="H102:H104"/>
+    <mergeCell ref="H105:H107"/>
+    <mergeCell ref="H108:H110"/>
+    <mergeCell ref="H111:H113"/>
+    <mergeCell ref="H114:H116"/>
+    <mergeCell ref="H117:H119"/>
+    <mergeCell ref="H125:H127"/>
+    <mergeCell ref="H63:H65"/>
+    <mergeCell ref="H66:H68"/>
+    <mergeCell ref="H69:H71"/>
+    <mergeCell ref="H72:H74"/>
+    <mergeCell ref="H75:H77"/>
+    <mergeCell ref="H78:H80"/>
+    <mergeCell ref="H84:H86"/>
+    <mergeCell ref="H81:H83"/>
+    <mergeCell ref="H87:H89"/>
+    <mergeCell ref="H36:H38"/>
+    <mergeCell ref="H39:H41"/>
+    <mergeCell ref="H42:H44"/>
+    <mergeCell ref="H45:H47"/>
+    <mergeCell ref="H48:H50"/>
+    <mergeCell ref="H51:H53"/>
+    <mergeCell ref="H54:H56"/>
+    <mergeCell ref="H57:H59"/>
+    <mergeCell ref="H60:H62"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="H18:H20"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="A84:A86"/>
+    <mergeCell ref="B84:B86"/>
+    <mergeCell ref="F84:F86"/>
+    <mergeCell ref="G84:G86"/>
+    <mergeCell ref="A57:A59"/>
+    <mergeCell ref="B57:B59"/>
+    <mergeCell ref="F57:F59"/>
+    <mergeCell ref="G57:G59"/>
+    <mergeCell ref="A69:A71"/>
+    <mergeCell ref="B69:B71"/>
+    <mergeCell ref="A72:A74"/>
+    <mergeCell ref="B72:B74"/>
+    <mergeCell ref="F69:F71"/>
+    <mergeCell ref="G69:G71"/>
+    <mergeCell ref="F72:F74"/>
+    <mergeCell ref="G72:G74"/>
+    <mergeCell ref="B63:B65"/>
+    <mergeCell ref="F63:F65"/>
+    <mergeCell ref="G63:G65"/>
+    <mergeCell ref="A66:A68"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="G66:G68"/>
+    <mergeCell ref="A75:A77"/>
+    <mergeCell ref="F60:F62"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="F75:F77"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="F33:F35"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="F42:F44"/>
+    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="G48:G50"/>
+    <mergeCell ref="F66:F68"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="F51:F53"/>
+    <mergeCell ref="G51:G53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="F54:F56"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="A60:A62"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="F39:F41"/>
+    <mergeCell ref="G39:G41"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="F45:F47"/>
+    <mergeCell ref="G45:G47"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="A93:A95"/>
+    <mergeCell ref="B93:B95"/>
+    <mergeCell ref="F93:F95"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="F48:F50"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="G93:G95"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="F30:F32"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="A78:A80"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="F78:F80"/>
+    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="A81:A83"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="F81:F83"/>
+    <mergeCell ref="G81:G83"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="F87:F89"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="A90:A92"/>
+    <mergeCell ref="B90:B92"/>
+    <mergeCell ref="F90:F92"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="F108:F110"/>
+    <mergeCell ref="G108:G110"/>
+    <mergeCell ref="A111:A113"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="F111:F113"/>
+    <mergeCell ref="G111:G113"/>
+    <mergeCell ref="A96:A98"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="F96:F98"/>
+    <mergeCell ref="G96:G98"/>
+    <mergeCell ref="A105:A107"/>
+    <mergeCell ref="B105:B107"/>
+    <mergeCell ref="F105:F107"/>
+    <mergeCell ref="G105:G107"/>
+    <mergeCell ref="G99:G101"/>
+    <mergeCell ref="A99:A101"/>
+    <mergeCell ref="B99:B101"/>
+    <mergeCell ref="F99:F101"/>
+    <mergeCell ref="A102:A104"/>
+    <mergeCell ref="B102:B104"/>
+    <mergeCell ref="F102:F104"/>
+    <mergeCell ref="G102:G104"/>
     <mergeCell ref="F120:F124"/>
     <mergeCell ref="G120:G124"/>
     <mergeCell ref="H120:H124"/>
@@ -3551,186 +3731,6 @@
     <mergeCell ref="C122:C124"/>
     <mergeCell ref="D122:D124"/>
     <mergeCell ref="E122:E124"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="F108:F110"/>
-    <mergeCell ref="G108:G110"/>
-    <mergeCell ref="A111:A113"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="F111:F113"/>
-    <mergeCell ref="G111:G113"/>
-    <mergeCell ref="A96:A98"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="F96:F98"/>
-    <mergeCell ref="G96:G98"/>
-    <mergeCell ref="A105:A107"/>
-    <mergeCell ref="B105:B107"/>
-    <mergeCell ref="F105:F107"/>
-    <mergeCell ref="G105:G107"/>
-    <mergeCell ref="G99:G101"/>
-    <mergeCell ref="A99:A101"/>
-    <mergeCell ref="B99:B101"/>
-    <mergeCell ref="F99:F101"/>
-    <mergeCell ref="A102:A104"/>
-    <mergeCell ref="B102:B104"/>
-    <mergeCell ref="F102:F104"/>
-    <mergeCell ref="G102:G104"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="G93:G95"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="F30:F32"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="A78:A80"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="F78:F80"/>
-    <mergeCell ref="G78:G80"/>
-    <mergeCell ref="A81:A83"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="F81:F83"/>
-    <mergeCell ref="G81:G83"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="F87:F89"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="A90:A92"/>
-    <mergeCell ref="B90:B92"/>
-    <mergeCell ref="F90:F92"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="A93:A95"/>
-    <mergeCell ref="B93:B95"/>
-    <mergeCell ref="F93:F95"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="F48:F50"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="F27:F29"/>
-    <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="A63:A65"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="F39:F41"/>
-    <mergeCell ref="G39:G41"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="F45:F47"/>
-    <mergeCell ref="G45:G47"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="F75:F77"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="F33:F35"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="F42:F44"/>
-    <mergeCell ref="G42:G44"/>
-    <mergeCell ref="G48:G50"/>
-    <mergeCell ref="F66:F68"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="F51:F53"/>
-    <mergeCell ref="G51:G53"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="F54:F56"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="A84:A86"/>
-    <mergeCell ref="B84:B86"/>
-    <mergeCell ref="F84:F86"/>
-    <mergeCell ref="G84:G86"/>
-    <mergeCell ref="A57:A59"/>
-    <mergeCell ref="B57:B59"/>
-    <mergeCell ref="F57:F59"/>
-    <mergeCell ref="G57:G59"/>
-    <mergeCell ref="A69:A71"/>
-    <mergeCell ref="B69:B71"/>
-    <mergeCell ref="A72:A74"/>
-    <mergeCell ref="B72:B74"/>
-    <mergeCell ref="F69:F71"/>
-    <mergeCell ref="G69:G71"/>
-    <mergeCell ref="F72:F74"/>
-    <mergeCell ref="G72:G74"/>
-    <mergeCell ref="B63:B65"/>
-    <mergeCell ref="F63:F65"/>
-    <mergeCell ref="G63:G65"/>
-    <mergeCell ref="A66:A68"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="G66:G68"/>
-    <mergeCell ref="A75:A77"/>
-    <mergeCell ref="F60:F62"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="H12:H14"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="H18:H20"/>
-    <mergeCell ref="H21:H23"/>
-    <mergeCell ref="H24:H26"/>
-    <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H35"/>
-    <mergeCell ref="H36:H38"/>
-    <mergeCell ref="H39:H41"/>
-    <mergeCell ref="H42:H44"/>
-    <mergeCell ref="H45:H47"/>
-    <mergeCell ref="H48:H50"/>
-    <mergeCell ref="H51:H53"/>
-    <mergeCell ref="H54:H56"/>
-    <mergeCell ref="H57:H59"/>
-    <mergeCell ref="H60:H62"/>
-    <mergeCell ref="H63:H65"/>
-    <mergeCell ref="H66:H68"/>
-    <mergeCell ref="H69:H71"/>
-    <mergeCell ref="H72:H74"/>
-    <mergeCell ref="H75:H77"/>
-    <mergeCell ref="H78:H80"/>
-    <mergeCell ref="H84:H86"/>
-    <mergeCell ref="H81:H83"/>
-    <mergeCell ref="H87:H89"/>
-    <mergeCell ref="H90:H92"/>
-    <mergeCell ref="H93:H95"/>
-    <mergeCell ref="H96:H98"/>
-    <mergeCell ref="H128:H130"/>
-    <mergeCell ref="H99:H101"/>
-    <mergeCell ref="H102:H104"/>
-    <mergeCell ref="H105:H107"/>
-    <mergeCell ref="H108:H110"/>
-    <mergeCell ref="H111:H113"/>
-    <mergeCell ref="H114:H116"/>
-    <mergeCell ref="H117:H119"/>
-    <mergeCell ref="H125:H127"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>

</xml_diff>

<commit_message>
Evidencias 28 de septiembre y 1 de octubre
</commit_message>
<xml_diff>
--- a/Cronograma/Itinerario-Ayo_Alisson V3.xlsx
+++ b/Cronograma/Itinerario-Ayo_Alisson V3.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MSI\Desktop\Prácticas\37009_PPP\Cronograma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9869C85-39E0-46EC-9244-8F4D8963318E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32E142C-2C51-4AA7-A249-831CA5D02BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -884,6 +884,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -911,15 +929,6 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -937,15 +946,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1240,15 +1240,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="24" x14ac:dyDescent="0.7">
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A2" s="4" t="s">
@@ -1316,10 +1316,10 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="33">
+      <c r="A9" s="26">
         <v>46279</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="26" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="14" t="s">
@@ -1329,17 +1329,17 @@
         <v>2</v>
       </c>
       <c r="E9" s="14"/>
-      <c r="F9" s="34" t="s">
+      <c r="F9" s="27" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="35">
-        <v>6</v>
-      </c>
-      <c r="H9" s="43"/>
+      <c r="G9" s="28">
+        <v>6</v>
+      </c>
+      <c r="H9" s="24"/>
     </row>
     <row r="10" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A10" s="33"/>
-      <c r="B10" s="33"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="26"/>
       <c r="C10" s="14" t="s">
         <v>19</v>
       </c>
@@ -1347,13 +1347,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="14"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="43"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="24"/>
     </row>
     <row r="11" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
       <c r="C11" s="14" t="s">
         <v>20</v>
       </c>
@@ -1364,15 +1364,15 @@
         <f>SUM(D9:D11)</f>
         <v>6</v>
       </c>
-      <c r="F11" s="34"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="43"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="24"/>
     </row>
     <row r="12" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A12" s="33">
+      <c r="A12" s="26">
         <v>46280</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="26" t="s">
         <v>22</v>
       </c>
       <c r="C12" s="14" t="s">
@@ -1382,17 +1382,17 @@
         <v>2</v>
       </c>
       <c r="E12" s="14"/>
-      <c r="F12" s="34" t="s">
+      <c r="F12" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="G12" s="35">
-        <v>6</v>
-      </c>
-      <c r="H12" s="43"/>
+      <c r="G12" s="28">
+        <v>6</v>
+      </c>
+      <c r="H12" s="24"/>
     </row>
     <row r="13" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A13" s="33"/>
-      <c r="B13" s="33"/>
+      <c r="A13" s="26"/>
+      <c r="B13" s="26"/>
       <c r="C13" s="14" t="s">
         <v>24</v>
       </c>
@@ -1400,13 +1400,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="13"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="43"/>
+      <c r="F13" s="27"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="24"/>
     </row>
     <row r="14" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A14" s="33"/>
-      <c r="B14" s="33"/>
+      <c r="A14" s="26"/>
+      <c r="B14" s="26"/>
       <c r="C14" s="14" t="s">
         <v>21</v>
       </c>
@@ -1416,15 +1416,15 @@
       <c r="E14" s="14">
         <v>6</v>
       </c>
-      <c r="F14" s="34"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="43"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="24"/>
     </row>
     <row r="15" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A15" s="33">
+      <c r="A15" s="26">
         <v>46281</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="26" t="s">
         <v>25</v>
       </c>
       <c r="C15" s="14" t="s">
@@ -1434,17 +1434,17 @@
         <v>2</v>
       </c>
       <c r="E15" s="13"/>
-      <c r="F15" s="34" t="s">
+      <c r="F15" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="35">
-        <v>6</v>
-      </c>
-      <c r="H15" s="43"/>
+      <c r="G15" s="28">
+        <v>6</v>
+      </c>
+      <c r="H15" s="24"/>
     </row>
     <row r="16" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A16" s="33"/>
-      <c r="B16" s="33"/>
+      <c r="A16" s="26"/>
+      <c r="B16" s="26"/>
       <c r="C16" s="20" t="s">
         <v>27</v>
       </c>
@@ -1452,13 +1452,13 @@
         <v>2</v>
       </c>
       <c r="E16" s="13"/>
-      <c r="F16" s="34"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="43"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A17" s="33"/>
-      <c r="B17" s="33"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="20" t="s">
         <v>28</v>
       </c>
@@ -1468,15 +1468,15 @@
       <c r="E17" s="14">
         <v>6</v>
       </c>
-      <c r="F17" s="34"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="43"/>
+      <c r="F17" s="27"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="24"/>
     </row>
     <row r="18" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A18" s="33">
+      <c r="A18" s="26">
         <v>46282</v>
       </c>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="26" t="s">
         <v>29</v>
       </c>
       <c r="C18" s="14" t="s">
@@ -1486,17 +1486,17 @@
         <v>2</v>
       </c>
       <c r="E18" s="13"/>
-      <c r="F18" s="34" t="s">
+      <c r="F18" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="35">
-        <v>6</v>
-      </c>
-      <c r="H18" s="43"/>
+      <c r="G18" s="28">
+        <v>6</v>
+      </c>
+      <c r="H18" s="24"/>
     </row>
     <row r="19" spans="1:8" ht="38.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="33"/>
-      <c r="B19" s="33"/>
+      <c r="A19" s="26"/>
+      <c r="B19" s="26"/>
       <c r="C19" s="14" t="s">
         <v>31</v>
       </c>
@@ -1504,13 +1504,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="13"/>
-      <c r="F19" s="34"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="43"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="24"/>
     </row>
     <row r="20" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A20" s="33"/>
-      <c r="B20" s="33"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="14" t="s">
         <v>32</v>
       </c>
@@ -1520,15 +1520,15 @@
       <c r="E20" s="14">
         <v>6</v>
       </c>
-      <c r="F20" s="34"/>
-      <c r="G20" s="35"/>
-      <c r="H20" s="43"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="28"/>
+      <c r="H20" s="24"/>
     </row>
     <row r="21" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A21" s="33">
+      <c r="A21" s="26">
         <v>46283</v>
       </c>
-      <c r="B21" s="33" t="s">
+      <c r="B21" s="26" t="s">
         <v>33</v>
       </c>
       <c r="C21" s="14" t="s">
@@ -1538,17 +1538,17 @@
         <v>2</v>
       </c>
       <c r="E21" s="13"/>
-      <c r="F21" s="34" t="s">
+      <c r="F21" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G21" s="35">
-        <v>6</v>
-      </c>
-      <c r="H21" s="43"/>
+      <c r="G21" s="28">
+        <v>6</v>
+      </c>
+      <c r="H21" s="24"/>
     </row>
     <row r="22" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A22" s="33"/>
-      <c r="B22" s="33"/>
+      <c r="A22" s="26"/>
+      <c r="B22" s="26"/>
       <c r="C22" s="14" t="s">
         <v>35</v>
       </c>
@@ -1556,13 +1556,13 @@
         <v>2</v>
       </c>
       <c r="E22" s="13"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="43"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="28"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A23" s="33"/>
-      <c r="B23" s="33"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="26"/>
       <c r="C23" s="14" t="s">
         <v>36</v>
       </c>
@@ -1572,15 +1572,15 @@
       <c r="E23" s="14">
         <v>6</v>
       </c>
-      <c r="F23" s="34"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="43"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="28"/>
+      <c r="H23" s="24"/>
     </row>
     <row r="24" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A24" s="33">
+      <c r="A24" s="26">
         <v>46286</v>
       </c>
-      <c r="B24" s="33" t="s">
+      <c r="B24" s="26" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="14" t="s">
@@ -1590,17 +1590,17 @@
         <v>2</v>
       </c>
       <c r="E24" s="14"/>
-      <c r="F24" s="34" t="s">
+      <c r="F24" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="G24" s="35">
-        <v>6</v>
-      </c>
-      <c r="H24" s="43"/>
+      <c r="G24" s="28">
+        <v>6</v>
+      </c>
+      <c r="H24" s="24"/>
     </row>
     <row r="25" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A25" s="33"/>
-      <c r="B25" s="33"/>
+      <c r="A25" s="26"/>
+      <c r="B25" s="26"/>
       <c r="C25" s="14" t="s">
         <v>39</v>
       </c>
@@ -1608,13 +1608,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="13"/>
-      <c r="F25" s="34"/>
-      <c r="G25" s="35"/>
-      <c r="H25" s="43"/>
+      <c r="F25" s="27"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="24"/>
     </row>
     <row r="26" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A26" s="33"/>
-      <c r="B26" s="33"/>
+      <c r="A26" s="26"/>
+      <c r="B26" s="26"/>
       <c r="C26" s="14" t="s">
         <v>40</v>
       </c>
@@ -1624,15 +1624,15 @@
       <c r="E26" s="14">
         <v>6</v>
       </c>
-      <c r="F26" s="34"/>
-      <c r="G26" s="35"/>
-      <c r="H26" s="43"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="24"/>
     </row>
     <row r="27" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A27" s="33">
+      <c r="A27" s="26">
         <v>46287</v>
       </c>
-      <c r="B27" s="33" t="s">
+      <c r="B27" s="26" t="s">
         <v>41</v>
       </c>
       <c r="C27" s="14" t="s">
@@ -1642,17 +1642,17 @@
         <v>2</v>
       </c>
       <c r="E27" s="13"/>
-      <c r="F27" s="34" t="s">
+      <c r="F27" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="35">
-        <v>6</v>
-      </c>
-      <c r="H27" s="43"/>
+      <c r="G27" s="28">
+        <v>6</v>
+      </c>
+      <c r="H27" s="24"/>
     </row>
     <row r="28" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A28" s="33"/>
-      <c r="B28" s="33"/>
+      <c r="A28" s="26"/>
+      <c r="B28" s="26"/>
       <c r="C28" s="14" t="s">
         <v>43</v>
       </c>
@@ -1660,13 +1660,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="13"/>
-      <c r="F28" s="34"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="43"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="24"/>
     </row>
     <row r="29" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A29" s="33"/>
-      <c r="B29" s="33"/>
+      <c r="A29" s="26"/>
+      <c r="B29" s="26"/>
       <c r="C29" s="14" t="s">
         <v>44</v>
       </c>
@@ -1676,15 +1676,15 @@
       <c r="E29" s="14">
         <v>6</v>
       </c>
-      <c r="F29" s="34"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="43"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="24"/>
     </row>
     <row r="30" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A30" s="33">
+      <c r="A30" s="26">
         <v>46288</v>
       </c>
-      <c r="B30" s="33" t="s">
+      <c r="B30" s="26" t="s">
         <v>45</v>
       </c>
       <c r="C30" s="14" t="s">
@@ -1694,17 +1694,17 @@
         <v>2</v>
       </c>
       <c r="E30" s="13"/>
-      <c r="F30" s="34" t="s">
+      <c r="F30" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="G30" s="35">
-        <v>6</v>
-      </c>
-      <c r="H30" s="43"/>
+      <c r="G30" s="28">
+        <v>6</v>
+      </c>
+      <c r="H30" s="24"/>
     </row>
     <row r="31" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A31" s="33"/>
-      <c r="B31" s="33"/>
+      <c r="A31" s="26"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="14" t="s">
         <v>47</v>
       </c>
@@ -1712,13 +1712,13 @@
         <v>2</v>
       </c>
       <c r="E31" s="13"/>
-      <c r="F31" s="34"/>
-      <c r="G31" s="35"/>
-      <c r="H31" s="43"/>
+      <c r="F31" s="27"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="24"/>
     </row>
     <row r="32" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A32" s="33"/>
-      <c r="B32" s="33"/>
+      <c r="A32" s="26"/>
+      <c r="B32" s="26"/>
       <c r="C32" s="14" t="s">
         <v>48</v>
       </c>
@@ -1728,15 +1728,15 @@
       <c r="E32" s="14">
         <v>6</v>
       </c>
-      <c r="F32" s="34"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="43"/>
+      <c r="F32" s="27"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="24"/>
     </row>
     <row r="33" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A33" s="33">
+      <c r="A33" s="26">
         <v>46289</v>
       </c>
-      <c r="B33" s="33" t="s">
+      <c r="B33" s="26" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="14" t="s">
@@ -1746,17 +1746,17 @@
         <v>2</v>
       </c>
       <c r="E33" s="13"/>
-      <c r="F33" s="34" t="s">
+      <c r="F33" s="27" t="s">
         <v>178</v>
       </c>
-      <c r="G33" s="35">
-        <v>6</v>
-      </c>
-      <c r="H33" s="43"/>
+      <c r="G33" s="28">
+        <v>6</v>
+      </c>
+      <c r="H33" s="24"/>
     </row>
     <row r="34" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A34" s="33"/>
-      <c r="B34" s="33"/>
+      <c r="A34" s="26"/>
+      <c r="B34" s="26"/>
       <c r="C34" s="14" t="s">
         <v>62</v>
       </c>
@@ -1764,13 +1764,13 @@
         <v>2</v>
       </c>
       <c r="E34" s="13"/>
-      <c r="F34" s="34"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="43"/>
+      <c r="F34" s="27"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="24"/>
     </row>
     <row r="35" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="33"/>
-      <c r="B35" s="33"/>
+      <c r="A35" s="26"/>
+      <c r="B35" s="26"/>
       <c r="C35" s="14" t="s">
         <v>63</v>
       </c>
@@ -1780,15 +1780,15 @@
       <c r="E35" s="14">
         <v>6</v>
       </c>
-      <c r="F35" s="34"/>
-      <c r="G35" s="35"/>
-      <c r="H35" s="43"/>
+      <c r="F35" s="27"/>
+      <c r="G35" s="28"/>
+      <c r="H35" s="24"/>
     </row>
     <row r="36" spans="1:8" ht="32.25" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A36" s="33">
+      <c r="A36" s="26">
         <v>46290</v>
       </c>
-      <c r="B36" s="33" t="s">
+      <c r="B36" s="26" t="s">
         <v>64</v>
       </c>
       <c r="C36" s="14" t="s">
@@ -1798,17 +1798,17 @@
         <v>2</v>
       </c>
       <c r="E36" s="14"/>
-      <c r="F36" s="34" t="s">
+      <c r="F36" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G36" s="35">
-        <v>6</v>
-      </c>
-      <c r="H36" s="43"/>
+      <c r="G36" s="28">
+        <v>6</v>
+      </c>
+      <c r="H36" s="24"/>
     </row>
     <row r="37" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A37" s="33"/>
-      <c r="B37" s="33"/>
+      <c r="A37" s="26"/>
+      <c r="B37" s="26"/>
       <c r="C37" s="14" t="s">
         <v>70</v>
       </c>
@@ -1816,13 +1816,13 @@
         <v>2</v>
       </c>
       <c r="E37" s="13"/>
-      <c r="F37" s="34"/>
-      <c r="G37" s="35"/>
-      <c r="H37" s="43"/>
+      <c r="F37" s="27"/>
+      <c r="G37" s="28"/>
+      <c r="H37" s="24"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A38" s="33"/>
-      <c r="B38" s="33"/>
+      <c r="A38" s="26"/>
+      <c r="B38" s="26"/>
       <c r="C38" s="14" t="s">
         <v>71</v>
       </c>
@@ -1832,15 +1832,15 @@
       <c r="E38" s="14">
         <v>6</v>
       </c>
-      <c r="F38" s="34"/>
-      <c r="G38" s="35"/>
-      <c r="H38" s="43"/>
+      <c r="F38" s="27"/>
+      <c r="G38" s="28"/>
+      <c r="H38" s="24"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A39" s="33">
+      <c r="A39" s="26">
         <v>46293</v>
       </c>
-      <c r="B39" s="33" t="s">
+      <c r="B39" s="26" t="s">
         <v>65</v>
       </c>
       <c r="C39" s="14" t="s">
@@ -1850,17 +1850,17 @@
         <v>2</v>
       </c>
       <c r="E39" s="13"/>
-      <c r="F39" s="34" t="s">
+      <c r="F39" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G39" s="35">
-        <v>6</v>
-      </c>
-      <c r="H39" s="43"/>
+      <c r="G39" s="28">
+        <v>6</v>
+      </c>
+      <c r="H39" s="24"/>
     </row>
     <row r="40" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A40" s="33"/>
-      <c r="B40" s="33"/>
+      <c r="A40" s="26"/>
+      <c r="B40" s="26"/>
       <c r="C40" s="14" t="s">
         <v>73</v>
       </c>
@@ -1868,13 +1868,13 @@
         <v>2</v>
       </c>
       <c r="E40" s="13"/>
-      <c r="F40" s="34"/>
-      <c r="G40" s="35"/>
-      <c r="H40" s="43"/>
+      <c r="F40" s="27"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="24"/>
     </row>
     <row r="41" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A41" s="33"/>
-      <c r="B41" s="33"/>
+      <c r="A41" s="26"/>
+      <c r="B41" s="26"/>
       <c r="C41" s="14" t="s">
         <v>74</v>
       </c>
@@ -1884,15 +1884,15 @@
       <c r="E41" s="14">
         <v>6</v>
       </c>
-      <c r="F41" s="34"/>
-      <c r="G41" s="35"/>
-      <c r="H41" s="43"/>
+      <c r="F41" s="27"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="24"/>
     </row>
     <row r="42" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A42" s="33">
+      <c r="A42" s="26">
         <v>46294</v>
       </c>
-      <c r="B42" s="33" t="s">
+      <c r="B42" s="26" t="s">
         <v>66</v>
       </c>
       <c r="C42" s="14" t="s">
@@ -1902,17 +1902,17 @@
         <v>2</v>
       </c>
       <c r="E42" s="13"/>
-      <c r="F42" s="34" t="s">
+      <c r="F42" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G42" s="35">
-        <v>6</v>
-      </c>
-      <c r="H42" s="43"/>
+      <c r="G42" s="28">
+        <v>6</v>
+      </c>
+      <c r="H42" s="24"/>
     </row>
     <row r="43" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A43" s="33"/>
-      <c r="B43" s="33"/>
+      <c r="A43" s="26"/>
+      <c r="B43" s="26"/>
       <c r="C43" s="14" t="s">
         <v>68</v>
       </c>
@@ -1920,13 +1920,13 @@
         <v>2</v>
       </c>
       <c r="E43" s="13"/>
-      <c r="F43" s="34"/>
-      <c r="G43" s="35"/>
-      <c r="H43" s="43"/>
+      <c r="F43" s="27"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="24"/>
     </row>
     <row r="44" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A44" s="33"/>
-      <c r="B44" s="33"/>
+      <c r="A44" s="26"/>
+      <c r="B44" s="26"/>
       <c r="C44" s="14" t="s">
         <v>76</v>
       </c>
@@ -1936,15 +1936,15 @@
       <c r="E44" s="14">
         <v>6</v>
       </c>
-      <c r="F44" s="34"/>
-      <c r="G44" s="35"/>
-      <c r="H44" s="43"/>
+      <c r="F44" s="27"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="24"/>
     </row>
     <row r="45" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A45" s="33">
+      <c r="A45" s="26">
         <v>46295</v>
       </c>
-      <c r="B45" s="33" t="s">
+      <c r="B45" s="26" t="s">
         <v>67</v>
       </c>
       <c r="C45" s="14" t="s">
@@ -1954,17 +1954,17 @@
         <v>2</v>
       </c>
       <c r="E45" s="13"/>
-      <c r="F45" s="34" t="s">
+      <c r="F45" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G45" s="35">
-        <v>6</v>
-      </c>
-      <c r="H45" s="43"/>
+      <c r="G45" s="28">
+        <v>6</v>
+      </c>
+      <c r="H45" s="24"/>
     </row>
     <row r="46" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A46" s="33"/>
-      <c r="B46" s="33"/>
+      <c r="A46" s="26"/>
+      <c r="B46" s="26"/>
       <c r="C46" s="14" t="s">
         <v>78</v>
       </c>
@@ -1972,13 +1972,13 @@
         <v>2</v>
       </c>
       <c r="E46" s="13"/>
-      <c r="F46" s="34"/>
-      <c r="G46" s="35"/>
-      <c r="H46" s="43"/>
+      <c r="F46" s="27"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="24"/>
     </row>
     <row r="47" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A47" s="33"/>
-      <c r="B47" s="33"/>
+      <c r="A47" s="26"/>
+      <c r="B47" s="26"/>
       <c r="C47" s="14" t="s">
         <v>79</v>
       </c>
@@ -1988,15 +1988,15 @@
       <c r="E47" s="14">
         <v>6</v>
       </c>
-      <c r="F47" s="34"/>
-      <c r="G47" s="35"/>
-      <c r="H47" s="43"/>
+      <c r="F47" s="27"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="24"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A48" s="33">
+      <c r="A48" s="26">
         <v>46296</v>
       </c>
-      <c r="B48" s="33" t="s">
+      <c r="B48" s="26" t="s">
         <v>80</v>
       </c>
       <c r="C48" s="14" t="s">
@@ -2006,17 +2006,17 @@
         <v>2</v>
       </c>
       <c r="E48" s="13"/>
-      <c r="F48" s="34" t="s">
+      <c r="F48" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G48" s="35">
-        <v>6</v>
-      </c>
-      <c r="H48" s="43"/>
+      <c r="G48" s="28">
+        <v>6</v>
+      </c>
+      <c r="H48" s="24"/>
     </row>
     <row r="49" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A49" s="33"/>
-      <c r="B49" s="33"/>
+      <c r="A49" s="26"/>
+      <c r="B49" s="26"/>
       <c r="C49" s="14" t="s">
         <v>82</v>
       </c>
@@ -2024,13 +2024,13 @@
         <v>2</v>
       </c>
       <c r="E49" s="13"/>
-      <c r="F49" s="34"/>
-      <c r="G49" s="35"/>
-      <c r="H49" s="43"/>
+      <c r="F49" s="27"/>
+      <c r="G49" s="28"/>
+      <c r="H49" s="24"/>
     </row>
     <row r="50" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A50" s="33"/>
-      <c r="B50" s="33"/>
+      <c r="A50" s="26"/>
+      <c r="B50" s="26"/>
       <c r="C50" s="14" t="s">
         <v>83</v>
       </c>
@@ -2040,15 +2040,15 @@
       <c r="E50" s="14">
         <v>6</v>
       </c>
-      <c r="F50" s="34"/>
-      <c r="G50" s="35"/>
-      <c r="H50" s="43"/>
+      <c r="F50" s="27"/>
+      <c r="G50" s="28"/>
+      <c r="H50" s="24"/>
     </row>
     <row r="51" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A51" s="33">
+      <c r="A51" s="26">
         <v>46297</v>
       </c>
-      <c r="B51" s="33" t="s">
+      <c r="B51" s="26" t="s">
         <v>84</v>
       </c>
       <c r="C51" s="14" t="s">
@@ -2058,17 +2058,17 @@
         <v>2</v>
       </c>
       <c r="E51" s="13"/>
-      <c r="F51" s="34" t="s">
+      <c r="F51" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G51" s="35">
-        <v>6</v>
-      </c>
-      <c r="H51" s="43"/>
+      <c r="G51" s="28">
+        <v>6</v>
+      </c>
+      <c r="H51" s="24"/>
     </row>
     <row r="52" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A52" s="33"/>
-      <c r="B52" s="33"/>
+      <c r="A52" s="26"/>
+      <c r="B52" s="26"/>
       <c r="C52" s="14" t="s">
         <v>86</v>
       </c>
@@ -2076,13 +2076,13 @@
         <v>2</v>
       </c>
       <c r="E52" s="13"/>
-      <c r="F52" s="34"/>
-      <c r="G52" s="35"/>
-      <c r="H52" s="43"/>
+      <c r="F52" s="27"/>
+      <c r="G52" s="28"/>
+      <c r="H52" s="24"/>
     </row>
     <row r="53" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A53" s="33"/>
-      <c r="B53" s="33"/>
+      <c r="A53" s="26"/>
+      <c r="B53" s="26"/>
       <c r="C53" s="14" t="s">
         <v>87</v>
       </c>
@@ -2092,15 +2092,15 @@
       <c r="E53" s="14">
         <v>6</v>
       </c>
-      <c r="F53" s="34"/>
-      <c r="G53" s="35"/>
-      <c r="H53" s="43"/>
+      <c r="F53" s="27"/>
+      <c r="G53" s="28"/>
+      <c r="H53" s="24"/>
     </row>
     <row r="54" spans="1:8" ht="30.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A54" s="33">
+      <c r="A54" s="26">
         <v>46300</v>
       </c>
-      <c r="B54" s="33" t="s">
+      <c r="B54" s="26" t="s">
         <v>88</v>
       </c>
       <c r="C54" s="14" t="s">
@@ -2110,17 +2110,17 @@
         <v>2</v>
       </c>
       <c r="E54" s="13"/>
-      <c r="F54" s="34" t="s">
+      <c r="F54" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G54" s="35">
-        <v>6</v>
-      </c>
-      <c r="H54" s="43"/>
+      <c r="G54" s="28">
+        <v>6</v>
+      </c>
+      <c r="H54" s="24"/>
     </row>
     <row r="55" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A55" s="33"/>
-      <c r="B55" s="33"/>
+      <c r="A55" s="26"/>
+      <c r="B55" s="26"/>
       <c r="C55" s="14" t="s">
         <v>90</v>
       </c>
@@ -2128,13 +2128,13 @@
         <v>2</v>
       </c>
       <c r="E55" s="13"/>
-      <c r="F55" s="34"/>
-      <c r="G55" s="35"/>
-      <c r="H55" s="43"/>
+      <c r="F55" s="27"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="24"/>
     </row>
     <row r="56" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A56" s="33"/>
-      <c r="B56" s="33"/>
+      <c r="A56" s="26"/>
+      <c r="B56" s="26"/>
       <c r="C56" s="14" t="s">
         <v>91</v>
       </c>
@@ -2144,15 +2144,15 @@
       <c r="E56" s="14">
         <v>6</v>
       </c>
-      <c r="F56" s="34"/>
-      <c r="G56" s="35"/>
-      <c r="H56" s="43"/>
+      <c r="F56" s="27"/>
+      <c r="G56" s="28"/>
+      <c r="H56" s="24"/>
     </row>
     <row r="57" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A57" s="33">
+      <c r="A57" s="26">
         <v>46301</v>
       </c>
-      <c r="B57" s="33" t="s">
+      <c r="B57" s="26" t="s">
         <v>92</v>
       </c>
       <c r="C57" s="14" t="s">
@@ -2162,17 +2162,17 @@
         <v>2</v>
       </c>
       <c r="E57" s="13"/>
-      <c r="F57" s="34" t="s">
+      <c r="F57" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G57" s="35">
-        <v>6</v>
-      </c>
-      <c r="H57" s="43"/>
+      <c r="G57" s="28">
+        <v>6</v>
+      </c>
+      <c r="H57" s="24"/>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="33"/>
-      <c r="B58" s="33"/>
+      <c r="A58" s="26"/>
+      <c r="B58" s="26"/>
       <c r="C58" s="14" t="s">
         <v>94</v>
       </c>
@@ -2180,13 +2180,13 @@
         <v>2</v>
       </c>
       <c r="E58" s="13"/>
-      <c r="F58" s="34"/>
-      <c r="G58" s="35"/>
-      <c r="H58" s="43"/>
+      <c r="F58" s="27"/>
+      <c r="G58" s="28"/>
+      <c r="H58" s="24"/>
     </row>
     <row r="59" spans="1:8" ht="34.799999999999997" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="33"/>
-      <c r="B59" s="33"/>
+      <c r="A59" s="26"/>
+      <c r="B59" s="26"/>
       <c r="C59" s="14" t="s">
         <v>95</v>
       </c>
@@ -2196,15 +2196,15 @@
       <c r="E59" s="14">
         <v>6</v>
       </c>
-      <c r="F59" s="34"/>
-      <c r="G59" s="35"/>
-      <c r="H59" s="43"/>
+      <c r="F59" s="27"/>
+      <c r="G59" s="28"/>
+      <c r="H59" s="24"/>
     </row>
     <row r="60" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A60" s="33">
+      <c r="A60" s="26">
         <v>46302</v>
       </c>
-      <c r="B60" s="33" t="s">
+      <c r="B60" s="26" t="s">
         <v>96</v>
       </c>
       <c r="C60" s="14" t="s">
@@ -2214,17 +2214,17 @@
         <v>2</v>
       </c>
       <c r="E60" s="13"/>
-      <c r="F60" s="34" t="s">
+      <c r="F60" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G60" s="35">
-        <v>6</v>
-      </c>
-      <c r="H60" s="43"/>
+      <c r="G60" s="28">
+        <v>6</v>
+      </c>
+      <c r="H60" s="24"/>
     </row>
     <row r="61" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A61" s="33"/>
-      <c r="B61" s="33"/>
+      <c r="A61" s="26"/>
+      <c r="B61" s="26"/>
       <c r="C61" s="14" t="s">
         <v>98</v>
       </c>
@@ -2232,13 +2232,13 @@
         <v>2</v>
       </c>
       <c r="E61" s="13"/>
-      <c r="F61" s="34"/>
-      <c r="G61" s="35"/>
-      <c r="H61" s="43"/>
+      <c r="F61" s="27"/>
+      <c r="G61" s="28"/>
+      <c r="H61" s="24"/>
     </row>
     <row r="62" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A62" s="33"/>
-      <c r="B62" s="33"/>
+      <c r="A62" s="26"/>
+      <c r="B62" s="26"/>
       <c r="C62" s="14" t="s">
         <v>99</v>
       </c>
@@ -2248,15 +2248,15 @@
       <c r="E62" s="14">
         <v>6</v>
       </c>
-      <c r="F62" s="34"/>
-      <c r="G62" s="35"/>
-      <c r="H62" s="43"/>
+      <c r="F62" s="27"/>
+      <c r="G62" s="28"/>
+      <c r="H62" s="24"/>
     </row>
     <row r="63" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A63" s="33">
+      <c r="A63" s="26">
         <v>46303</v>
       </c>
-      <c r="B63" s="33" t="s">
+      <c r="B63" s="26" t="s">
         <v>100</v>
       </c>
       <c r="C63" s="14" t="s">
@@ -2266,17 +2266,17 @@
         <v>2</v>
       </c>
       <c r="E63" s="13"/>
-      <c r="F63" s="34" t="s">
+      <c r="F63" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G63" s="35">
-        <v>6</v>
-      </c>
-      <c r="H63" s="43"/>
+      <c r="G63" s="28">
+        <v>6</v>
+      </c>
+      <c r="H63" s="24"/>
     </row>
     <row r="64" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A64" s="33"/>
-      <c r="B64" s="33"/>
+      <c r="A64" s="26"/>
+      <c r="B64" s="26"/>
       <c r="C64" s="14" t="s">
         <v>102</v>
       </c>
@@ -2284,13 +2284,13 @@
         <v>2</v>
       </c>
       <c r="E64" s="13"/>
-      <c r="F64" s="34"/>
-      <c r="G64" s="35"/>
-      <c r="H64" s="43"/>
+      <c r="F64" s="27"/>
+      <c r="G64" s="28"/>
+      <c r="H64" s="24"/>
     </row>
     <row r="65" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A65" s="33"/>
-      <c r="B65" s="33"/>
+      <c r="A65" s="26"/>
+      <c r="B65" s="26"/>
       <c r="C65" s="14" t="s">
         <v>173</v>
       </c>
@@ -2300,15 +2300,15 @@
       <c r="E65" s="14">
         <v>6</v>
       </c>
-      <c r="F65" s="34"/>
-      <c r="G65" s="35"/>
-      <c r="H65" s="43"/>
+      <c r="F65" s="27"/>
+      <c r="G65" s="28"/>
+      <c r="H65" s="24"/>
     </row>
     <row r="66" spans="1:8" ht="28.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="33">
+      <c r="A66" s="26">
         <v>46307</v>
       </c>
-      <c r="B66" s="33" t="s">
+      <c r="B66" s="26" t="s">
         <v>103</v>
       </c>
       <c r="C66" s="14" t="s">
@@ -2318,17 +2318,17 @@
         <v>2</v>
       </c>
       <c r="E66" s="13"/>
-      <c r="F66" s="34" t="s">
+      <c r="F66" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G66" s="35">
-        <v>6</v>
-      </c>
-      <c r="H66" s="43"/>
+      <c r="G66" s="28">
+        <v>6</v>
+      </c>
+      <c r="H66" s="24"/>
     </row>
     <row r="67" spans="1:8" ht="32.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A67" s="33"/>
-      <c r="B67" s="33"/>
+      <c r="A67" s="26"/>
+      <c r="B67" s="26"/>
       <c r="C67" s="14" t="s">
         <v>106</v>
       </c>
@@ -2336,13 +2336,13 @@
         <v>2</v>
       </c>
       <c r="E67" s="14"/>
-      <c r="F67" s="34"/>
-      <c r="G67" s="35"/>
-      <c r="H67" s="43"/>
+      <c r="F67" s="27"/>
+      <c r="G67" s="28"/>
+      <c r="H67" s="24"/>
     </row>
     <row r="68" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A68" s="33"/>
-      <c r="B68" s="33"/>
+      <c r="A68" s="26"/>
+      <c r="B68" s="26"/>
       <c r="C68" s="14" t="s">
         <v>107</v>
       </c>
@@ -2352,15 +2352,15 @@
       <c r="E68" s="14">
         <v>6</v>
       </c>
-      <c r="F68" s="34"/>
-      <c r="G68" s="35"/>
-      <c r="H68" s="43"/>
+      <c r="F68" s="27"/>
+      <c r="G68" s="28"/>
+      <c r="H68" s="24"/>
     </row>
     <row r="69" spans="1:8" ht="54" x14ac:dyDescent="0.5">
-      <c r="A69" s="33">
+      <c r="A69" s="26">
         <v>46308</v>
       </c>
-      <c r="B69" s="35" t="s">
+      <c r="B69" s="28" t="s">
         <v>104</v>
       </c>
       <c r="C69" s="14" t="s">
@@ -2370,17 +2370,17 @@
         <v>2</v>
       </c>
       <c r="E69" s="14"/>
-      <c r="F69" s="34" t="s">
+      <c r="F69" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G69" s="35">
-        <v>6</v>
-      </c>
-      <c r="H69" s="43"/>
+      <c r="G69" s="28">
+        <v>6</v>
+      </c>
+      <c r="H69" s="24"/>
     </row>
     <row r="70" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A70" s="33"/>
-      <c r="B70" s="35"/>
+      <c r="A70" s="26"/>
+      <c r="B70" s="28"/>
       <c r="C70" s="14" t="s">
         <v>108</v>
       </c>
@@ -2388,13 +2388,13 @@
         <v>2</v>
       </c>
       <c r="E70" s="14"/>
-      <c r="F70" s="34"/>
-      <c r="G70" s="35"/>
-      <c r="H70" s="43"/>
+      <c r="F70" s="27"/>
+      <c r="G70" s="28"/>
+      <c r="H70" s="24"/>
     </row>
     <row r="71" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A71" s="33"/>
-      <c r="B71" s="35"/>
+      <c r="A71" s="26"/>
+      <c r="B71" s="28"/>
       <c r="C71" s="14" t="s">
         <v>143</v>
       </c>
@@ -2404,15 +2404,15 @@
       <c r="E71" s="14">
         <v>6</v>
       </c>
-      <c r="F71" s="34"/>
-      <c r="G71" s="35"/>
-      <c r="H71" s="43"/>
+      <c r="F71" s="27"/>
+      <c r="G71" s="28"/>
+      <c r="H71" s="24"/>
     </row>
     <row r="72" spans="1:8" ht="31.8" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="33">
+      <c r="A72" s="26">
         <v>46309</v>
       </c>
-      <c r="B72" s="35" t="s">
+      <c r="B72" s="28" t="s">
         <v>109</v>
       </c>
       <c r="C72" s="14" t="s">
@@ -2422,17 +2422,17 @@
         <v>2</v>
       </c>
       <c r="E72" s="14"/>
-      <c r="F72" s="34" t="s">
+      <c r="F72" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G72" s="35">
-        <v>6</v>
-      </c>
-      <c r="H72" s="43"/>
+      <c r="G72" s="28">
+        <v>6</v>
+      </c>
+      <c r="H72" s="24"/>
     </row>
     <row r="73" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A73" s="33"/>
-      <c r="B73" s="35"/>
+      <c r="A73" s="26"/>
+      <c r="B73" s="28"/>
       <c r="C73" s="14" t="s">
         <v>110</v>
       </c>
@@ -2440,13 +2440,13 @@
         <v>2</v>
       </c>
       <c r="E73" s="14"/>
-      <c r="F73" s="34"/>
-      <c r="G73" s="35"/>
-      <c r="H73" s="43"/>
+      <c r="F73" s="27"/>
+      <c r="G73" s="28"/>
+      <c r="H73" s="24"/>
     </row>
     <row r="74" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A74" s="33"/>
-      <c r="B74" s="35"/>
+      <c r="A74" s="26"/>
+      <c r="B74" s="28"/>
       <c r="C74" s="14" t="s">
         <v>111</v>
       </c>
@@ -2456,15 +2456,15 @@
       <c r="E74" s="14">
         <v>6</v>
       </c>
-      <c r="F74" s="34"/>
-      <c r="G74" s="35"/>
-      <c r="H74" s="43"/>
+      <c r="F74" s="27"/>
+      <c r="G74" s="28"/>
+      <c r="H74" s="24"/>
     </row>
     <row r="75" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A75" s="33">
+      <c r="A75" s="26">
         <v>46310</v>
       </c>
-      <c r="B75" s="35" t="s">
+      <c r="B75" s="28" t="s">
         <v>49</v>
       </c>
       <c r="C75" s="14" t="s">
@@ -2474,17 +2474,17 @@
         <v>2</v>
       </c>
       <c r="E75" s="14"/>
-      <c r="F75" s="34" t="s">
+      <c r="F75" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G75" s="35">
-        <v>6</v>
-      </c>
-      <c r="H75" s="43"/>
+      <c r="G75" s="28">
+        <v>6</v>
+      </c>
+      <c r="H75" s="24"/>
     </row>
     <row r="76" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A76" s="33"/>
-      <c r="B76" s="35"/>
+      <c r="A76" s="26"/>
+      <c r="B76" s="28"/>
       <c r="C76" s="14" t="s">
         <v>113</v>
       </c>
@@ -2492,13 +2492,13 @@
         <v>2</v>
       </c>
       <c r="E76" s="14"/>
-      <c r="F76" s="34"/>
-      <c r="G76" s="35"/>
-      <c r="H76" s="43"/>
+      <c r="F76" s="27"/>
+      <c r="G76" s="28"/>
+      <c r="H76" s="24"/>
     </row>
     <row r="77" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A77" s="33"/>
-      <c r="B77" s="35"/>
+      <c r="A77" s="26"/>
+      <c r="B77" s="28"/>
       <c r="C77" s="14" t="s">
         <v>114</v>
       </c>
@@ -2508,15 +2508,15 @@
       <c r="E77" s="14">
         <v>6</v>
       </c>
-      <c r="F77" s="34"/>
-      <c r="G77" s="35"/>
-      <c r="H77" s="43"/>
+      <c r="F77" s="27"/>
+      <c r="G77" s="28"/>
+      <c r="H77" s="24"/>
     </row>
     <row r="78" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A78" s="33">
+      <c r="A78" s="26">
         <v>46311</v>
       </c>
-      <c r="B78" s="33" t="s">
+      <c r="B78" s="26" t="s">
         <v>49</v>
       </c>
       <c r="C78" s="14" t="s">
@@ -2526,17 +2526,17 @@
         <v>2</v>
       </c>
       <c r="E78" s="14"/>
-      <c r="F78" s="34" t="s">
+      <c r="F78" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G78" s="35">
-        <v>6</v>
-      </c>
-      <c r="H78" s="43"/>
+      <c r="G78" s="28">
+        <v>6</v>
+      </c>
+      <c r="H78" s="24"/>
     </row>
     <row r="79" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A79" s="33"/>
-      <c r="B79" s="33"/>
+      <c r="A79" s="26"/>
+      <c r="B79" s="26"/>
       <c r="C79" s="14" t="s">
         <v>116</v>
       </c>
@@ -2544,13 +2544,13 @@
         <v>2</v>
       </c>
       <c r="E79" s="14"/>
-      <c r="F79" s="34"/>
-      <c r="G79" s="35"/>
-      <c r="H79" s="43"/>
+      <c r="F79" s="27"/>
+      <c r="G79" s="28"/>
+      <c r="H79" s="24"/>
     </row>
     <row r="80" spans="1:8" ht="33.6" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A80" s="33"/>
-      <c r="B80" s="33"/>
+      <c r="A80" s="26"/>
+      <c r="B80" s="26"/>
       <c r="C80" s="14" t="s">
         <v>117</v>
       </c>
@@ -2560,15 +2560,15 @@
       <c r="E80" s="14">
         <v>6</v>
       </c>
-      <c r="F80" s="34"/>
-      <c r="G80" s="35"/>
-      <c r="H80" s="43"/>
+      <c r="F80" s="27"/>
+      <c r="G80" s="28"/>
+      <c r="H80" s="24"/>
     </row>
     <row r="81" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A81" s="33">
+      <c r="A81" s="26">
         <v>46314</v>
       </c>
-      <c r="B81" s="33" t="s">
+      <c r="B81" s="26" t="s">
         <v>118</v>
       </c>
       <c r="C81" s="20" t="s">
@@ -2578,17 +2578,17 @@
         <v>2</v>
       </c>
       <c r="E81" s="14"/>
-      <c r="F81" s="34" t="s">
+      <c r="F81" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G81" s="35">
-        <v>6</v>
-      </c>
-      <c r="H81" s="44"/>
+      <c r="G81" s="28">
+        <v>6</v>
+      </c>
+      <c r="H81" s="25"/>
     </row>
     <row r="82" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A82" s="33"/>
-      <c r="B82" s="33"/>
+      <c r="A82" s="26"/>
+      <c r="B82" s="26"/>
       <c r="C82" s="20" t="s">
         <v>120</v>
       </c>
@@ -2596,13 +2596,13 @@
         <v>2</v>
       </c>
       <c r="E82" s="14"/>
-      <c r="F82" s="34"/>
-      <c r="G82" s="35"/>
-      <c r="H82" s="44"/>
+      <c r="F82" s="27"/>
+      <c r="G82" s="28"/>
+      <c r="H82" s="25"/>
     </row>
     <row r="83" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A83" s="33"/>
-      <c r="B83" s="33"/>
+      <c r="A83" s="26"/>
+      <c r="B83" s="26"/>
       <c r="C83" s="14" t="s">
         <v>121</v>
       </c>
@@ -2612,15 +2612,15 @@
       <c r="E83" s="14">
         <v>6</v>
       </c>
-      <c r="F83" s="34"/>
-      <c r="G83" s="35"/>
-      <c r="H83" s="44"/>
+      <c r="F83" s="27"/>
+      <c r="G83" s="28"/>
+      <c r="H83" s="25"/>
     </row>
     <row r="84" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A84" s="33">
+      <c r="A84" s="26">
         <v>46315</v>
       </c>
-      <c r="B84" s="33" t="s">
+      <c r="B84" s="26" t="s">
         <v>50</v>
       </c>
       <c r="C84" s="14" t="s">
@@ -2630,17 +2630,17 @@
         <v>2</v>
       </c>
       <c r="E84" s="14"/>
-      <c r="F84" s="34" t="s">
+      <c r="F84" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G84" s="35">
-        <v>6</v>
-      </c>
-      <c r="H84" s="43"/>
+      <c r="G84" s="28">
+        <v>6</v>
+      </c>
+      <c r="H84" s="24"/>
     </row>
     <row r="85" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A85" s="33"/>
-      <c r="B85" s="33"/>
+      <c r="A85" s="26"/>
+      <c r="B85" s="26"/>
       <c r="C85" s="14" t="s">
         <v>123</v>
       </c>
@@ -2648,13 +2648,13 @@
         <v>2</v>
       </c>
       <c r="E85" s="14"/>
-      <c r="F85" s="34"/>
-      <c r="G85" s="35"/>
-      <c r="H85" s="43"/>
+      <c r="F85" s="27"/>
+      <c r="G85" s="28"/>
+      <c r="H85" s="24"/>
     </row>
     <row r="86" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A86" s="33"/>
-      <c r="B86" s="33"/>
+      <c r="A86" s="26"/>
+      <c r="B86" s="26"/>
       <c r="C86" s="20" t="s">
         <v>124</v>
       </c>
@@ -2664,15 +2664,15 @@
       <c r="E86" s="14">
         <v>6</v>
       </c>
-      <c r="F86" s="34"/>
-      <c r="G86" s="35"/>
-      <c r="H86" s="43"/>
+      <c r="F86" s="27"/>
+      <c r="G86" s="28"/>
+      <c r="H86" s="24"/>
     </row>
     <row r="87" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A87" s="33">
+      <c r="A87" s="26">
         <v>46316</v>
       </c>
-      <c r="B87" s="33" t="s">
+      <c r="B87" s="26" t="s">
         <v>50</v>
       </c>
       <c r="C87" s="14" t="s">
@@ -2682,17 +2682,17 @@
         <v>2</v>
       </c>
       <c r="E87" s="14"/>
-      <c r="F87" s="34" t="s">
+      <c r="F87" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G87" s="35">
-        <v>6</v>
-      </c>
-      <c r="H87" s="43"/>
+      <c r="G87" s="28">
+        <v>6</v>
+      </c>
+      <c r="H87" s="24"/>
     </row>
     <row r="88" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A88" s="33"/>
-      <c r="B88" s="33"/>
+      <c r="A88" s="26"/>
+      <c r="B88" s="26"/>
       <c r="C88" s="14" t="s">
         <v>126</v>
       </c>
@@ -2700,13 +2700,13 @@
         <v>2</v>
       </c>
       <c r="E88" s="13"/>
-      <c r="F88" s="34"/>
-      <c r="G88" s="35"/>
-      <c r="H88" s="43"/>
+      <c r="F88" s="27"/>
+      <c r="G88" s="28"/>
+      <c r="H88" s="24"/>
     </row>
     <row r="89" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A89" s="33"/>
-      <c r="B89" s="33"/>
+      <c r="A89" s="26"/>
+      <c r="B89" s="26"/>
       <c r="C89" s="14" t="s">
         <v>127</v>
       </c>
@@ -2716,15 +2716,15 @@
       <c r="E89" s="14">
         <v>6</v>
       </c>
-      <c r="F89" s="34"/>
-      <c r="G89" s="35"/>
-      <c r="H89" s="43"/>
+      <c r="F89" s="27"/>
+      <c r="G89" s="28"/>
+      <c r="H89" s="24"/>
     </row>
     <row r="90" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A90" s="33">
+      <c r="A90" s="26">
         <v>46317</v>
       </c>
-      <c r="B90" s="35" t="s">
+      <c r="B90" s="28" t="s">
         <v>130</v>
       </c>
       <c r="C90" s="14" t="s">
@@ -2734,17 +2734,17 @@
         <v>2</v>
       </c>
       <c r="E90" s="13"/>
-      <c r="F90" s="34" t="s">
+      <c r="F90" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G90" s="35">
-        <v>6</v>
-      </c>
-      <c r="H90" s="43"/>
+      <c r="G90" s="28">
+        <v>6</v>
+      </c>
+      <c r="H90" s="24"/>
     </row>
     <row r="91" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A91" s="33"/>
-      <c r="B91" s="35"/>
+      <c r="A91" s="26"/>
+      <c r="B91" s="28"/>
       <c r="C91" s="14" t="s">
         <v>120</v>
       </c>
@@ -2752,13 +2752,13 @@
         <v>2</v>
       </c>
       <c r="E91" s="13"/>
-      <c r="F91" s="34"/>
-      <c r="G91" s="35"/>
-      <c r="H91" s="43"/>
+      <c r="F91" s="27"/>
+      <c r="G91" s="28"/>
+      <c r="H91" s="24"/>
     </row>
     <row r="92" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A92" s="33"/>
-      <c r="B92" s="35"/>
+      <c r="A92" s="26"/>
+      <c r="B92" s="28"/>
       <c r="C92" s="14" t="s">
         <v>129</v>
       </c>
@@ -2768,15 +2768,15 @@
       <c r="E92" s="14">
         <v>6</v>
       </c>
-      <c r="F92" s="34"/>
-      <c r="G92" s="35"/>
-      <c r="H92" s="43"/>
+      <c r="F92" s="27"/>
+      <c r="G92" s="28"/>
+      <c r="H92" s="24"/>
     </row>
     <row r="93" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A93" s="33">
+      <c r="A93" s="26">
         <v>46318</v>
       </c>
-      <c r="B93" s="35" t="s">
+      <c r="B93" s="28" t="s">
         <v>51</v>
       </c>
       <c r="C93" s="20" t="s">
@@ -2786,17 +2786,17 @@
         <v>2</v>
       </c>
       <c r="E93" s="13"/>
-      <c r="F93" s="34" t="s">
+      <c r="F93" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G93" s="35">
-        <v>6</v>
-      </c>
-      <c r="H93" s="43"/>
+      <c r="G93" s="28">
+        <v>6</v>
+      </c>
+      <c r="H93" s="24"/>
     </row>
     <row r="94" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A94" s="33"/>
-      <c r="B94" s="35"/>
+      <c r="A94" s="26"/>
+      <c r="B94" s="28"/>
       <c r="C94" s="20" t="s">
         <v>132</v>
       </c>
@@ -2804,13 +2804,13 @@
         <v>2</v>
       </c>
       <c r="E94" s="13"/>
-      <c r="F94" s="34"/>
-      <c r="G94" s="35"/>
-      <c r="H94" s="43"/>
+      <c r="F94" s="27"/>
+      <c r="G94" s="28"/>
+      <c r="H94" s="24"/>
     </row>
     <row r="95" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A95" s="33"/>
-      <c r="B95" s="35"/>
+      <c r="A95" s="26"/>
+      <c r="B95" s="28"/>
       <c r="C95" s="14" t="s">
         <v>133</v>
       </c>
@@ -2820,15 +2820,15 @@
       <c r="E95" s="14">
         <v>6</v>
       </c>
-      <c r="F95" s="34"/>
-      <c r="G95" s="35"/>
-      <c r="H95" s="43"/>
+      <c r="F95" s="27"/>
+      <c r="G95" s="28"/>
+      <c r="H95" s="24"/>
     </row>
     <row r="96" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A96" s="33">
+      <c r="A96" s="26">
         <v>46321</v>
       </c>
-      <c r="B96" s="35" t="s">
+      <c r="B96" s="28" t="s">
         <v>51</v>
       </c>
       <c r="C96" s="14" t="s">
@@ -2838,17 +2838,17 @@
         <v>2</v>
       </c>
       <c r="E96" s="14"/>
-      <c r="F96" s="34" t="s">
+      <c r="F96" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G96" s="35">
-        <v>6</v>
-      </c>
-      <c r="H96" s="43"/>
+      <c r="G96" s="28">
+        <v>6</v>
+      </c>
+      <c r="H96" s="24"/>
     </row>
     <row r="97" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A97" s="33"/>
-      <c r="B97" s="35"/>
+      <c r="A97" s="26"/>
+      <c r="B97" s="28"/>
       <c r="C97" s="20" t="s">
         <v>135</v>
       </c>
@@ -2856,13 +2856,13 @@
         <v>2</v>
       </c>
       <c r="E97" s="13"/>
-      <c r="F97" s="34"/>
-      <c r="G97" s="35"/>
-      <c r="H97" s="43"/>
+      <c r="F97" s="27"/>
+      <c r="G97" s="28"/>
+      <c r="H97" s="24"/>
     </row>
     <row r="98" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A98" s="33"/>
-      <c r="B98" s="35"/>
+      <c r="A98" s="26"/>
+      <c r="B98" s="28"/>
       <c r="C98" s="14" t="s">
         <v>136</v>
       </c>
@@ -2872,15 +2872,15 @@
       <c r="E98" s="14">
         <v>6</v>
       </c>
-      <c r="F98" s="34"/>
-      <c r="G98" s="35"/>
-      <c r="H98" s="43"/>
+      <c r="F98" s="27"/>
+      <c r="G98" s="28"/>
+      <c r="H98" s="24"/>
     </row>
     <row r="99" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A99" s="33">
+      <c r="A99" s="26">
         <v>46322</v>
       </c>
-      <c r="B99" s="35" t="s">
+      <c r="B99" s="28" t="s">
         <v>137</v>
       </c>
       <c r="C99" s="14" t="s">
@@ -2890,17 +2890,17 @@
         <v>2</v>
       </c>
       <c r="E99" s="13"/>
-      <c r="F99" s="34" t="s">
+      <c r="F99" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G99" s="35">
-        <v>6</v>
-      </c>
-      <c r="H99" s="43"/>
+      <c r="G99" s="28">
+        <v>6</v>
+      </c>
+      <c r="H99" s="24"/>
     </row>
     <row r="100" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A100" s="33"/>
-      <c r="B100" s="35"/>
+      <c r="A100" s="26"/>
+      <c r="B100" s="28"/>
       <c r="C100" s="14" t="s">
         <v>120</v>
       </c>
@@ -2908,13 +2908,13 @@
         <v>2</v>
       </c>
       <c r="E100" s="13"/>
-      <c r="F100" s="34"/>
-      <c r="G100" s="35"/>
-      <c r="H100" s="43"/>
+      <c r="F100" s="27"/>
+      <c r="G100" s="28"/>
+      <c r="H100" s="24"/>
     </row>
     <row r="101" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A101" s="33"/>
-      <c r="B101" s="35"/>
+      <c r="A101" s="26"/>
+      <c r="B101" s="28"/>
       <c r="C101" s="14" t="s">
         <v>139</v>
       </c>
@@ -2924,15 +2924,15 @@
       <c r="E101" s="14">
         <v>6</v>
       </c>
-      <c r="F101" s="34"/>
-      <c r="G101" s="35"/>
-      <c r="H101" s="43"/>
+      <c r="F101" s="27"/>
+      <c r="G101" s="28"/>
+      <c r="H101" s="24"/>
     </row>
     <row r="102" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A102" s="33">
+      <c r="A102" s="26">
         <v>46323</v>
       </c>
-      <c r="B102" s="35" t="s">
+      <c r="B102" s="28" t="s">
         <v>140</v>
       </c>
       <c r="C102" s="14" t="s">
@@ -2942,17 +2942,17 @@
         <v>2</v>
       </c>
       <c r="E102" s="14"/>
-      <c r="F102" s="34" t="s">
+      <c r="F102" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G102" s="35">
-        <v>6</v>
-      </c>
-      <c r="H102" s="43"/>
+      <c r="G102" s="28">
+        <v>6</v>
+      </c>
+      <c r="H102" s="24"/>
     </row>
     <row r="103" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A103" s="33"/>
-      <c r="B103" s="35"/>
+      <c r="A103" s="26"/>
+      <c r="B103" s="28"/>
       <c r="C103" s="20" t="s">
         <v>142</v>
       </c>
@@ -2960,13 +2960,13 @@
         <v>2</v>
       </c>
       <c r="E103" s="13"/>
-      <c r="F103" s="34"/>
-      <c r="G103" s="35"/>
-      <c r="H103" s="43"/>
+      <c r="F103" s="27"/>
+      <c r="G103" s="28"/>
+      <c r="H103" s="24"/>
     </row>
     <row r="104" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A104" s="33"/>
-      <c r="B104" s="35"/>
+      <c r="A104" s="26"/>
+      <c r="B104" s="28"/>
       <c r="C104" s="14" t="s">
         <v>144</v>
       </c>
@@ -2976,15 +2976,15 @@
       <c r="E104" s="14">
         <v>6</v>
       </c>
-      <c r="F104" s="34"/>
-      <c r="G104" s="35"/>
-      <c r="H104" s="43"/>
+      <c r="F104" s="27"/>
+      <c r="G104" s="28"/>
+      <c r="H104" s="24"/>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A105" s="33">
+      <c r="A105" s="26">
         <v>46324</v>
       </c>
-      <c r="B105" s="34" t="s">
+      <c r="B105" s="27" t="s">
         <v>145</v>
       </c>
       <c r="C105" s="14" t="s">
@@ -2994,17 +2994,17 @@
         <v>2</v>
       </c>
       <c r="E105" s="13"/>
-      <c r="F105" s="34" t="s">
+      <c r="F105" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G105" s="35">
-        <v>6</v>
-      </c>
-      <c r="H105" s="43"/>
+      <c r="G105" s="28">
+        <v>6</v>
+      </c>
+      <c r="H105" s="24"/>
     </row>
     <row r="106" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A106" s="33"/>
-      <c r="B106" s="34"/>
+      <c r="A106" s="26"/>
+      <c r="B106" s="27"/>
       <c r="C106" s="14" t="s">
         <v>147</v>
       </c>
@@ -3012,13 +3012,13 @@
         <v>2</v>
       </c>
       <c r="E106" s="13"/>
-      <c r="F106" s="34"/>
-      <c r="G106" s="35"/>
-      <c r="H106" s="43"/>
+      <c r="F106" s="27"/>
+      <c r="G106" s="28"/>
+      <c r="H106" s="24"/>
     </row>
     <row r="107" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A107" s="33"/>
-      <c r="B107" s="34"/>
+      <c r="A107" s="26"/>
+      <c r="B107" s="27"/>
       <c r="C107" s="14" t="s">
         <v>148</v>
       </c>
@@ -3028,15 +3028,15 @@
       <c r="E107" s="14">
         <v>6</v>
       </c>
-      <c r="F107" s="34"/>
-      <c r="G107" s="35"/>
-      <c r="H107" s="43"/>
+      <c r="F107" s="27"/>
+      <c r="G107" s="28"/>
+      <c r="H107" s="24"/>
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A108" s="33">
+      <c r="A108" s="26">
         <v>46325</v>
       </c>
-      <c r="B108" s="34" t="s">
+      <c r="B108" s="27" t="s">
         <v>149</v>
       </c>
       <c r="C108" s="14" t="s">
@@ -3046,17 +3046,17 @@
         <v>2</v>
       </c>
       <c r="E108" s="13"/>
-      <c r="F108" s="34" t="s">
+      <c r="F108" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G108" s="35">
-        <v>6</v>
-      </c>
-      <c r="H108" s="43"/>
+      <c r="G108" s="28">
+        <v>6</v>
+      </c>
+      <c r="H108" s="24"/>
     </row>
     <row r="109" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A109" s="33"/>
-      <c r="B109" s="34"/>
+      <c r="A109" s="26"/>
+      <c r="B109" s="27"/>
       <c r="C109" s="15" t="s">
         <v>151</v>
       </c>
@@ -3064,13 +3064,13 @@
         <v>2</v>
       </c>
       <c r="E109" s="13"/>
-      <c r="F109" s="34"/>
-      <c r="G109" s="35"/>
-      <c r="H109" s="43"/>
+      <c r="F109" s="27"/>
+      <c r="G109" s="28"/>
+      <c r="H109" s="24"/>
     </row>
     <row r="110" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A110" s="33"/>
-      <c r="B110" s="34"/>
+      <c r="A110" s="26"/>
+      <c r="B110" s="27"/>
       <c r="C110" s="14" t="s">
         <v>152</v>
       </c>
@@ -3080,15 +3080,15 @@
       <c r="E110" s="14">
         <v>6</v>
       </c>
-      <c r="F110" s="34"/>
-      <c r="G110" s="35"/>
-      <c r="H110" s="43"/>
+      <c r="F110" s="27"/>
+      <c r="G110" s="28"/>
+      <c r="H110" s="24"/>
     </row>
     <row r="111" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A111" s="33">
+      <c r="A111" s="26">
         <v>46330</v>
       </c>
-      <c r="B111" s="34" t="s">
+      <c r="B111" s="27" t="s">
         <v>153</v>
       </c>
       <c r="C111" s="14" t="s">
@@ -3098,17 +3098,17 @@
         <v>2</v>
       </c>
       <c r="E111" s="13"/>
-      <c r="F111" s="34" t="s">
+      <c r="F111" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G111" s="35">
-        <v>6</v>
-      </c>
-      <c r="H111" s="43"/>
+      <c r="G111" s="28">
+        <v>6</v>
+      </c>
+      <c r="H111" s="24"/>
     </row>
     <row r="112" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A112" s="33"/>
-      <c r="B112" s="34"/>
+      <c r="A112" s="26"/>
+      <c r="B112" s="27"/>
       <c r="C112" s="14" t="s">
         <v>155</v>
       </c>
@@ -3116,13 +3116,13 @@
         <v>2</v>
       </c>
       <c r="E112" s="13"/>
-      <c r="F112" s="34"/>
-      <c r="G112" s="35"/>
-      <c r="H112" s="43"/>
+      <c r="F112" s="27"/>
+      <c r="G112" s="28"/>
+      <c r="H112" s="24"/>
     </row>
     <row r="113" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A113" s="33"/>
-      <c r="B113" s="34"/>
+      <c r="A113" s="26"/>
+      <c r="B113" s="27"/>
       <c r="C113" s="14" t="s">
         <v>156</v>
       </c>
@@ -3132,15 +3132,15 @@
       <c r="E113" s="14">
         <v>6</v>
       </c>
-      <c r="F113" s="34"/>
-      <c r="G113" s="35"/>
-      <c r="H113" s="43"/>
+      <c r="F113" s="27"/>
+      <c r="G113" s="28"/>
+      <c r="H113" s="24"/>
     </row>
     <row r="114" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A114" s="33">
+      <c r="A114" s="26">
         <v>46331</v>
       </c>
-      <c r="B114" s="34" t="s">
+      <c r="B114" s="27" t="s">
         <v>157</v>
       </c>
       <c r="C114" s="14" t="s">
@@ -3150,17 +3150,17 @@
         <v>2</v>
       </c>
       <c r="E114" s="13"/>
-      <c r="F114" s="34" t="s">
+      <c r="F114" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G114" s="35">
-        <v>6</v>
-      </c>
-      <c r="H114" s="43"/>
+      <c r="G114" s="28">
+        <v>6</v>
+      </c>
+      <c r="H114" s="24"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A115" s="33"/>
-      <c r="B115" s="34"/>
+      <c r="A115" s="26"/>
+      <c r="B115" s="27"/>
       <c r="C115" s="14" t="s">
         <v>159</v>
       </c>
@@ -3168,13 +3168,13 @@
         <v>2</v>
       </c>
       <c r="E115" s="13"/>
-      <c r="F115" s="34"/>
-      <c r="G115" s="35"/>
-      <c r="H115" s="43"/>
+      <c r="F115" s="27"/>
+      <c r="G115" s="28"/>
+      <c r="H115" s="24"/>
     </row>
     <row r="116" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A116" s="33"/>
-      <c r="B116" s="34"/>
+      <c r="A116" s="26"/>
+      <c r="B116" s="27"/>
       <c r="C116" s="14" t="s">
         <v>160</v>
       </c>
@@ -3184,15 +3184,15 @@
       <c r="E116" s="14">
         <v>6</v>
       </c>
-      <c r="F116" s="34"/>
-      <c r="G116" s="35"/>
-      <c r="H116" s="43"/>
+      <c r="F116" s="27"/>
+      <c r="G116" s="28"/>
+      <c r="H116" s="24"/>
     </row>
     <row r="117" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A117" s="33">
+      <c r="A117" s="26">
         <v>46332</v>
       </c>
-      <c r="B117" s="34" t="s">
+      <c r="B117" s="27" t="s">
         <v>161</v>
       </c>
       <c r="C117" s="14" t="s">
@@ -3202,17 +3202,17 @@
         <v>2</v>
       </c>
       <c r="E117" s="13"/>
-      <c r="F117" s="34" t="s">
+      <c r="F117" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G117" s="35">
-        <v>6</v>
-      </c>
-      <c r="H117" s="43"/>
+      <c r="G117" s="28">
+        <v>6</v>
+      </c>
+      <c r="H117" s="24"/>
     </row>
     <row r="118" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A118" s="33"/>
-      <c r="B118" s="34"/>
+      <c r="A118" s="26"/>
+      <c r="B118" s="27"/>
       <c r="C118" s="14" t="s">
         <v>163</v>
       </c>
@@ -3220,13 +3220,13 @@
         <v>2</v>
       </c>
       <c r="E118" s="13"/>
-      <c r="F118" s="34"/>
-      <c r="G118" s="35"/>
-      <c r="H118" s="43"/>
+      <c r="F118" s="27"/>
+      <c r="G118" s="28"/>
+      <c r="H118" s="24"/>
     </row>
     <row r="119" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A119" s="33"/>
-      <c r="B119" s="34"/>
+      <c r="A119" s="26"/>
+      <c r="B119" s="27"/>
       <c r="C119" s="14" t="s">
         <v>176</v>
       </c>
@@ -3236,15 +3236,15 @@
       <c r="E119" s="14">
         <v>6</v>
       </c>
-      <c r="F119" s="34"/>
-      <c r="G119" s="35"/>
-      <c r="H119" s="43"/>
+      <c r="F119" s="27"/>
+      <c r="G119" s="28"/>
+      <c r="H119" s="24"/>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A120" s="36">
+      <c r="A120" s="39">
         <v>46335</v>
       </c>
-      <c r="B120" s="24" t="s">
+      <c r="B120" s="30" t="s">
         <v>164</v>
       </c>
       <c r="C120" s="22" t="s">
@@ -3254,17 +3254,17 @@
         <v>2</v>
       </c>
       <c r="E120" s="22"/>
-      <c r="F120" s="24" t="s">
+      <c r="F120" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="G120" s="27">
-        <v>6</v>
-      </c>
-      <c r="H120" s="30"/>
+      <c r="G120" s="33">
+        <v>6</v>
+      </c>
+      <c r="H120" s="36"/>
     </row>
     <row r="121" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A121" s="37"/>
-      <c r="B121" s="25"/>
+      <c r="A121" s="40"/>
+      <c r="B121" s="31"/>
       <c r="C121" s="22" t="s">
         <v>166</v>
       </c>
@@ -3272,51 +3272,51 @@
         <v>2</v>
       </c>
       <c r="E121" s="22"/>
-      <c r="F121" s="25"/>
-      <c r="G121" s="28"/>
-      <c r="H121" s="31"/>
+      <c r="F121" s="31"/>
+      <c r="G121" s="34"/>
+      <c r="H121" s="37"/>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A122" s="37"/>
-      <c r="B122" s="25"/>
-      <c r="C122" s="24" t="s">
+      <c r="A122" s="40"/>
+      <c r="B122" s="31"/>
+      <c r="C122" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="D122" s="39">
-        <v>2</v>
-      </c>
-      <c r="E122" s="39">
-        <v>6</v>
-      </c>
-      <c r="F122" s="25"/>
-      <c r="G122" s="28"/>
-      <c r="H122" s="31"/>
+      <c r="D122" s="42">
+        <v>2</v>
+      </c>
+      <c r="E122" s="42">
+        <v>6</v>
+      </c>
+      <c r="F122" s="31"/>
+      <c r="G122" s="34"/>
+      <c r="H122" s="37"/>
     </row>
     <row r="123" spans="1:8" ht="11.4" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A123" s="37"/>
-      <c r="B123" s="25"/>
-      <c r="C123" s="25"/>
-      <c r="D123" s="40"/>
-      <c r="E123" s="40"/>
-      <c r="F123" s="25"/>
-      <c r="G123" s="28"/>
-      <c r="H123" s="31"/>
+      <c r="A123" s="40"/>
+      <c r="B123" s="31"/>
+      <c r="C123" s="31"/>
+      <c r="D123" s="43"/>
+      <c r="E123" s="43"/>
+      <c r="F123" s="31"/>
+      <c r="G123" s="34"/>
+      <c r="H123" s="37"/>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A124" s="38"/>
-      <c r="B124" s="26"/>
-      <c r="C124" s="26"/>
-      <c r="D124" s="41"/>
-      <c r="E124" s="41"/>
-      <c r="F124" s="26"/>
-      <c r="G124" s="29"/>
-      <c r="H124" s="32"/>
+      <c r="A124" s="41"/>
+      <c r="B124" s="32"/>
+      <c r="C124" s="32"/>
+      <c r="D124" s="44"/>
+      <c r="E124" s="44"/>
+      <c r="F124" s="32"/>
+      <c r="G124" s="35"/>
+      <c r="H124" s="38"/>
     </row>
     <row r="125" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A125" s="33">
+      <c r="A125" s="26">
         <v>46336</v>
       </c>
-      <c r="B125" s="34" t="s">
+      <c r="B125" s="27" t="s">
         <v>168</v>
       </c>
       <c r="C125" s="14" t="s">
@@ -3326,17 +3326,17 @@
         <v>2</v>
       </c>
       <c r="E125" s="13"/>
-      <c r="F125" s="34" t="s">
+      <c r="F125" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G125" s="35">
-        <v>6</v>
-      </c>
-      <c r="H125" s="43"/>
+      <c r="G125" s="28">
+        <v>6</v>
+      </c>
+      <c r="H125" s="24"/>
     </row>
     <row r="126" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A126" s="33"/>
-      <c r="B126" s="34"/>
+      <c r="A126" s="26"/>
+      <c r="B126" s="27"/>
       <c r="C126" s="14" t="s">
         <v>169</v>
       </c>
@@ -3344,13 +3344,13 @@
         <v>2</v>
       </c>
       <c r="E126" s="13"/>
-      <c r="F126" s="34"/>
-      <c r="G126" s="35"/>
-      <c r="H126" s="43"/>
+      <c r="F126" s="27"/>
+      <c r="G126" s="28"/>
+      <c r="H126" s="24"/>
     </row>
     <row r="127" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A127" s="33"/>
-      <c r="B127" s="34"/>
+      <c r="A127" s="26"/>
+      <c r="B127" s="27"/>
       <c r="C127" s="14" t="s">
         <v>170</v>
       </c>
@@ -3360,15 +3360,15 @@
       <c r="E127" s="14">
         <v>6</v>
       </c>
-      <c r="F127" s="34"/>
-      <c r="G127" s="35"/>
-      <c r="H127" s="43"/>
+      <c r="F127" s="27"/>
+      <c r="G127" s="28"/>
+      <c r="H127" s="24"/>
     </row>
     <row r="128" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A128" s="33">
+      <c r="A128" s="26">
         <v>46337</v>
       </c>
-      <c r="B128" s="34" t="s">
+      <c r="B128" s="27" t="s">
         <v>52</v>
       </c>
       <c r="C128" s="14" t="s">
@@ -3378,17 +3378,17 @@
         <v>2</v>
       </c>
       <c r="E128" s="13"/>
-      <c r="F128" s="34" t="s">
+      <c r="F128" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="G128" s="35">
-        <v>6</v>
-      </c>
-      <c r="H128" s="43"/>
+      <c r="G128" s="28">
+        <v>6</v>
+      </c>
+      <c r="H128" s="24"/>
     </row>
     <row r="129" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A129" s="33"/>
-      <c r="B129" s="34"/>
+      <c r="A129" s="26"/>
+      <c r="B129" s="27"/>
       <c r="C129" s="14" t="s">
         <v>172</v>
       </c>
@@ -3396,13 +3396,13 @@
         <v>2</v>
       </c>
       <c r="E129" s="13"/>
-      <c r="F129" s="34"/>
-      <c r="G129" s="35"/>
-      <c r="H129" s="43"/>
+      <c r="F129" s="27"/>
+      <c r="G129" s="28"/>
+      <c r="H129" s="24"/>
     </row>
     <row r="130" spans="1:8" ht="36" x14ac:dyDescent="0.5">
-      <c r="A130" s="33"/>
-      <c r="B130" s="34"/>
+      <c r="A130" s="26"/>
+      <c r="B130" s="27"/>
       <c r="C130" s="14" t="s">
         <v>53</v>
       </c>
@@ -3412,9 +3412,9 @@
       <c r="E130" s="14">
         <v>6</v>
       </c>
-      <c r="F130" s="34"/>
-      <c r="G130" s="35"/>
-      <c r="H130" s="43"/>
+      <c r="F130" s="27"/>
+      <c r="G130" s="28"/>
+      <c r="H130" s="24"/>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A131" s="11"/>
@@ -3527,45 +3527,147 @@
     </row>
   </sheetData>
   <mergeCells count="204">
-    <mergeCell ref="H90:H92"/>
-    <mergeCell ref="H93:H95"/>
-    <mergeCell ref="H96:H98"/>
-    <mergeCell ref="H128:H130"/>
-    <mergeCell ref="H99:H101"/>
-    <mergeCell ref="H102:H104"/>
-    <mergeCell ref="H105:H107"/>
-    <mergeCell ref="H108:H110"/>
-    <mergeCell ref="H111:H113"/>
-    <mergeCell ref="H114:H116"/>
-    <mergeCell ref="H117:H119"/>
-    <mergeCell ref="H125:H127"/>
-    <mergeCell ref="H63:H65"/>
-    <mergeCell ref="H66:H68"/>
-    <mergeCell ref="H69:H71"/>
-    <mergeCell ref="H72:H74"/>
-    <mergeCell ref="H75:H77"/>
-    <mergeCell ref="H78:H80"/>
-    <mergeCell ref="H84:H86"/>
-    <mergeCell ref="H81:H83"/>
-    <mergeCell ref="H87:H89"/>
-    <mergeCell ref="H36:H38"/>
-    <mergeCell ref="H39:H41"/>
-    <mergeCell ref="H42:H44"/>
-    <mergeCell ref="H45:H47"/>
-    <mergeCell ref="H48:H50"/>
-    <mergeCell ref="H51:H53"/>
-    <mergeCell ref="H54:H56"/>
-    <mergeCell ref="H57:H59"/>
-    <mergeCell ref="H60:H62"/>
-    <mergeCell ref="H9:H11"/>
-    <mergeCell ref="H12:H14"/>
-    <mergeCell ref="H15:H17"/>
-    <mergeCell ref="H18:H20"/>
-    <mergeCell ref="H21:H23"/>
-    <mergeCell ref="H24:H26"/>
-    <mergeCell ref="H27:H29"/>
-    <mergeCell ref="H30:H32"/>
-    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="F120:F124"/>
+    <mergeCell ref="G120:G124"/>
+    <mergeCell ref="H120:H124"/>
+    <mergeCell ref="A114:A116"/>
+    <mergeCell ref="B114:B116"/>
+    <mergeCell ref="F114:F116"/>
+    <mergeCell ref="A128:A130"/>
+    <mergeCell ref="B128:B130"/>
+    <mergeCell ref="F128:F130"/>
+    <mergeCell ref="G128:G130"/>
+    <mergeCell ref="A117:A119"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="F117:F119"/>
+    <mergeCell ref="G117:G119"/>
+    <mergeCell ref="A125:A127"/>
+    <mergeCell ref="B125:B127"/>
+    <mergeCell ref="F125:F127"/>
+    <mergeCell ref="G125:G127"/>
+    <mergeCell ref="G114:G116"/>
+    <mergeCell ref="A120:A124"/>
+    <mergeCell ref="B120:B124"/>
+    <mergeCell ref="C122:C124"/>
+    <mergeCell ref="D122:D124"/>
+    <mergeCell ref="E122:E124"/>
+    <mergeCell ref="A108:A110"/>
+    <mergeCell ref="B108:B110"/>
+    <mergeCell ref="F108:F110"/>
+    <mergeCell ref="G108:G110"/>
+    <mergeCell ref="A111:A113"/>
+    <mergeCell ref="B111:B113"/>
+    <mergeCell ref="F111:F113"/>
+    <mergeCell ref="G111:G113"/>
+    <mergeCell ref="A96:A98"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="F96:F98"/>
+    <mergeCell ref="G96:G98"/>
+    <mergeCell ref="A105:A107"/>
+    <mergeCell ref="B105:B107"/>
+    <mergeCell ref="F105:F107"/>
+    <mergeCell ref="G105:G107"/>
+    <mergeCell ref="G99:G101"/>
+    <mergeCell ref="A99:A101"/>
+    <mergeCell ref="B99:B101"/>
+    <mergeCell ref="F99:F101"/>
+    <mergeCell ref="A102:A104"/>
+    <mergeCell ref="B102:B104"/>
+    <mergeCell ref="F102:F104"/>
+    <mergeCell ref="G102:G104"/>
+    <mergeCell ref="F12:F14"/>
+    <mergeCell ref="G12:G14"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="A12:A14"/>
+    <mergeCell ref="B24:B26"/>
+    <mergeCell ref="A24:A26"/>
+    <mergeCell ref="F24:F26"/>
+    <mergeCell ref="G24:G26"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="G93:G95"/>
+    <mergeCell ref="A45:A47"/>
+    <mergeCell ref="B45:B47"/>
+    <mergeCell ref="F36:F38"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="A30:A32"/>
+    <mergeCell ref="B30:B32"/>
+    <mergeCell ref="F30:F32"/>
+    <mergeCell ref="G30:G32"/>
+    <mergeCell ref="A78:A80"/>
+    <mergeCell ref="B78:B80"/>
+    <mergeCell ref="F78:F80"/>
+    <mergeCell ref="G78:G80"/>
+    <mergeCell ref="A81:A83"/>
+    <mergeCell ref="B81:B83"/>
+    <mergeCell ref="F81:F83"/>
+    <mergeCell ref="G81:G83"/>
+    <mergeCell ref="A87:A89"/>
+    <mergeCell ref="B87:B89"/>
+    <mergeCell ref="F87:F89"/>
+    <mergeCell ref="G87:G89"/>
+    <mergeCell ref="A90:A92"/>
+    <mergeCell ref="B90:B92"/>
+    <mergeCell ref="F90:F92"/>
+    <mergeCell ref="G90:G92"/>
+    <mergeCell ref="A93:A95"/>
+    <mergeCell ref="B93:B95"/>
+    <mergeCell ref="F93:F95"/>
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B9:B11"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="G9:G11"/>
+    <mergeCell ref="A48:A50"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="F48:F50"/>
+    <mergeCell ref="A15:A17"/>
+    <mergeCell ref="B15:B17"/>
+    <mergeCell ref="F15:F17"/>
+    <mergeCell ref="G15:G17"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="A21:A23"/>
+    <mergeCell ref="B21:B23"/>
+    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="G21:G23"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="B27:B29"/>
+    <mergeCell ref="F27:F29"/>
+    <mergeCell ref="G27:G29"/>
+    <mergeCell ref="G60:G62"/>
+    <mergeCell ref="A63:A65"/>
+    <mergeCell ref="B42:B44"/>
+    <mergeCell ref="A42:A44"/>
+    <mergeCell ref="A39:A41"/>
+    <mergeCell ref="B39:B41"/>
+    <mergeCell ref="F39:F41"/>
+    <mergeCell ref="G39:G41"/>
+    <mergeCell ref="B60:B62"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="F45:F47"/>
+    <mergeCell ref="G45:G47"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="F75:F77"/>
+    <mergeCell ref="G75:G77"/>
+    <mergeCell ref="A33:A35"/>
+    <mergeCell ref="B33:B35"/>
+    <mergeCell ref="F33:F35"/>
+    <mergeCell ref="G33:G35"/>
+    <mergeCell ref="F42:F44"/>
+    <mergeCell ref="G42:G44"/>
+    <mergeCell ref="G48:G50"/>
+    <mergeCell ref="F66:F68"/>
+    <mergeCell ref="A51:A53"/>
+    <mergeCell ref="B51:B53"/>
+    <mergeCell ref="F51:F53"/>
+    <mergeCell ref="G51:G53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="F54:F56"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="A60:A62"/>
     <mergeCell ref="A84:A86"/>
     <mergeCell ref="B84:B86"/>
     <mergeCell ref="F84:F86"/>
@@ -3590,147 +3692,45 @@
     <mergeCell ref="G66:G68"/>
     <mergeCell ref="A75:A77"/>
     <mergeCell ref="F60:F62"/>
-    <mergeCell ref="B75:B77"/>
-    <mergeCell ref="F75:F77"/>
-    <mergeCell ref="G75:G77"/>
-    <mergeCell ref="A33:A35"/>
-    <mergeCell ref="B33:B35"/>
-    <mergeCell ref="F33:F35"/>
-    <mergeCell ref="G33:G35"/>
-    <mergeCell ref="F42:F44"/>
-    <mergeCell ref="G42:G44"/>
-    <mergeCell ref="G48:G50"/>
-    <mergeCell ref="F66:F68"/>
-    <mergeCell ref="A51:A53"/>
-    <mergeCell ref="B51:B53"/>
-    <mergeCell ref="F51:F53"/>
-    <mergeCell ref="G51:G53"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="F54:F56"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="A60:A62"/>
-    <mergeCell ref="G27:G29"/>
-    <mergeCell ref="G60:G62"/>
-    <mergeCell ref="A63:A65"/>
-    <mergeCell ref="B42:B44"/>
-    <mergeCell ref="A42:A44"/>
-    <mergeCell ref="A39:A41"/>
-    <mergeCell ref="B39:B41"/>
-    <mergeCell ref="F39:F41"/>
-    <mergeCell ref="G39:G41"/>
-    <mergeCell ref="B60:B62"/>
-    <mergeCell ref="A36:A38"/>
-    <mergeCell ref="B36:B38"/>
-    <mergeCell ref="F45:F47"/>
-    <mergeCell ref="G45:G47"/>
-    <mergeCell ref="G90:G92"/>
-    <mergeCell ref="A93:A95"/>
-    <mergeCell ref="B93:B95"/>
-    <mergeCell ref="F93:F95"/>
-    <mergeCell ref="B1:H1"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="A9:A11"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="G9:G11"/>
-    <mergeCell ref="A48:A50"/>
-    <mergeCell ref="B48:B50"/>
-    <mergeCell ref="F48:F50"/>
-    <mergeCell ref="A15:A17"/>
-    <mergeCell ref="B15:B17"/>
-    <mergeCell ref="F15:F17"/>
-    <mergeCell ref="G15:G17"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="A21:A23"/>
-    <mergeCell ref="B21:B23"/>
-    <mergeCell ref="F21:F23"/>
-    <mergeCell ref="G21:G23"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="B27:B29"/>
-    <mergeCell ref="F27:F29"/>
-    <mergeCell ref="G93:G95"/>
-    <mergeCell ref="A45:A47"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="F36:F38"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="F30:F32"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="A78:A80"/>
-    <mergeCell ref="B78:B80"/>
-    <mergeCell ref="F78:F80"/>
-    <mergeCell ref="G78:G80"/>
-    <mergeCell ref="A81:A83"/>
-    <mergeCell ref="B81:B83"/>
-    <mergeCell ref="F81:F83"/>
-    <mergeCell ref="G81:G83"/>
-    <mergeCell ref="A87:A89"/>
-    <mergeCell ref="B87:B89"/>
-    <mergeCell ref="F87:F89"/>
-    <mergeCell ref="G87:G89"/>
-    <mergeCell ref="A90:A92"/>
-    <mergeCell ref="B90:B92"/>
-    <mergeCell ref="F90:F92"/>
-    <mergeCell ref="F12:F14"/>
-    <mergeCell ref="G12:G14"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A108:A110"/>
-    <mergeCell ref="B108:B110"/>
-    <mergeCell ref="F108:F110"/>
-    <mergeCell ref="G108:G110"/>
-    <mergeCell ref="A111:A113"/>
-    <mergeCell ref="B111:B113"/>
-    <mergeCell ref="F111:F113"/>
-    <mergeCell ref="G111:G113"/>
-    <mergeCell ref="A96:A98"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="F96:F98"/>
-    <mergeCell ref="G96:G98"/>
-    <mergeCell ref="A105:A107"/>
-    <mergeCell ref="B105:B107"/>
-    <mergeCell ref="F105:F107"/>
-    <mergeCell ref="G105:G107"/>
-    <mergeCell ref="G99:G101"/>
-    <mergeCell ref="A99:A101"/>
-    <mergeCell ref="B99:B101"/>
-    <mergeCell ref="F99:F101"/>
-    <mergeCell ref="A102:A104"/>
-    <mergeCell ref="B102:B104"/>
-    <mergeCell ref="F102:F104"/>
-    <mergeCell ref="G102:G104"/>
-    <mergeCell ref="F120:F124"/>
-    <mergeCell ref="G120:G124"/>
-    <mergeCell ref="H120:H124"/>
-    <mergeCell ref="A114:A116"/>
-    <mergeCell ref="B114:B116"/>
-    <mergeCell ref="F114:F116"/>
-    <mergeCell ref="A128:A130"/>
-    <mergeCell ref="B128:B130"/>
-    <mergeCell ref="F128:F130"/>
-    <mergeCell ref="G128:G130"/>
-    <mergeCell ref="A117:A119"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="F117:F119"/>
-    <mergeCell ref="G117:G119"/>
-    <mergeCell ref="A125:A127"/>
-    <mergeCell ref="B125:B127"/>
-    <mergeCell ref="F125:F127"/>
-    <mergeCell ref="G125:G127"/>
-    <mergeCell ref="G114:G116"/>
-    <mergeCell ref="A120:A124"/>
-    <mergeCell ref="B120:B124"/>
-    <mergeCell ref="C122:C124"/>
-    <mergeCell ref="D122:D124"/>
-    <mergeCell ref="E122:E124"/>
+    <mergeCell ref="H9:H11"/>
+    <mergeCell ref="H12:H14"/>
+    <mergeCell ref="H15:H17"/>
+    <mergeCell ref="H18:H20"/>
+    <mergeCell ref="H21:H23"/>
+    <mergeCell ref="H24:H26"/>
+    <mergeCell ref="H27:H29"/>
+    <mergeCell ref="H30:H32"/>
+    <mergeCell ref="H33:H35"/>
+    <mergeCell ref="H36:H38"/>
+    <mergeCell ref="H39:H41"/>
+    <mergeCell ref="H42:H44"/>
+    <mergeCell ref="H45:H47"/>
+    <mergeCell ref="H48:H50"/>
+    <mergeCell ref="H51:H53"/>
+    <mergeCell ref="H54:H56"/>
+    <mergeCell ref="H57:H59"/>
+    <mergeCell ref="H60:H62"/>
+    <mergeCell ref="H63:H65"/>
+    <mergeCell ref="H66:H68"/>
+    <mergeCell ref="H69:H71"/>
+    <mergeCell ref="H72:H74"/>
+    <mergeCell ref="H75:H77"/>
+    <mergeCell ref="H78:H80"/>
+    <mergeCell ref="H84:H86"/>
+    <mergeCell ref="H81:H83"/>
+    <mergeCell ref="H87:H89"/>
+    <mergeCell ref="H90:H92"/>
+    <mergeCell ref="H93:H95"/>
+    <mergeCell ref="H96:H98"/>
+    <mergeCell ref="H128:H130"/>
+    <mergeCell ref="H99:H101"/>
+    <mergeCell ref="H102:H104"/>
+    <mergeCell ref="H105:H107"/>
+    <mergeCell ref="H108:H110"/>
+    <mergeCell ref="H111:H113"/>
+    <mergeCell ref="H114:H116"/>
+    <mergeCell ref="H117:H119"/>
+    <mergeCell ref="H125:H127"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="3" orientation="landscape" r:id="rId1"/>

</xml_diff>